<commit_message>
Modified to support admin mode.
</commit_message>
<xml_diff>
--- a/tools/template.xlsx
+++ b/tools/template.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V399"/>
+  <dimension ref="A1:X399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -468,8 +468,10 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="52" customWidth="1" min="19" max="19"/>
     <col width="52" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="52" customWidth="1" min="21" max="21"/>
+    <col width="52" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -575,10 +577,20 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
+          <t>insight_en</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>insight_th</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>ref</t>
         </is>
@@ -663,12 +675,14 @@
           <t>ส่วนที่ยังเหลืออยู่หลังใส่มาตรการควบคุมแล้วคือความเสี่ยงคงเหลือ</t>
         </is>
       </c>
-      <c r="U2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr"/>
+      <c r="V2" s="3" t="inlineStr"/>
+      <c r="W2" s="3" t="inlineStr">
         <is>
           <t>risk-management</t>
         </is>
       </c>
-      <c r="V2" s="3" t="inlineStr"/>
+      <c r="X2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr"/>
@@ -749,36 +763,113 @@
           <t>CIA triad ประกอบด้วย Confidentiality, Integrity และ Availability</t>
         </is>
       </c>
-      <c r="U3" s="3" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr"/>
+      <c r="V3" s="3" t="inlineStr"/>
+      <c r="W3" s="3" t="inlineStr">
         <is>
           <t>fundamentals</t>
         </is>
       </c>
-      <c r="V3" s="3" t="inlineStr"/>
+      <c r="X3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3" t="n"/>
-      <c r="R4" s="3" t="n"/>
-      <c r="S4" s="3" t="n"/>
-      <c r="T4" s="3" t="n"/>
-      <c r="U4" s="3" t="n"/>
-      <c r="V4" s="3" t="n"/>
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Alyssa is responsible for her organization's security awareness program. She is concerned that changes in technology may make the content outdated.
+What control can she put in place to protect against this risk?</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Alyssa รับผิดชอบโปรแกรมสร้างตระหนักรู้ด้านความมั่นคงปลอดภัย (security awareness program) ขององค์กร เธอมีความกังวลว่าการเปลี่ยนแปลงทางเทคโนโลยีอาจทำให้เนื้อหาฝึกอบรมล้าสมัย
+มาตรการควบคุม (control) ใดที่เธอสามารถนำมาใช้เพื่อป้องกันความเสี่ยงนี้ได้?</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Gamification</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Gamification (การใช้เทคนิคเกมในการอบรม)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Computer-based training</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Computer-based training (การฝึกอบรมผ่านคอมพิวเตอร์)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Content Reviews</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Content Reviews (การทบทวนและตรวจสอบเนื้อหา)</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Live training</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Live training (การฝึกอบรมแบบสด/มีวิทยากร)</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="3" t="inlineStr"/>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>Alyssa should use periodic content reviews to continually verify that the content in her program meets the organization's needs and is up-to-date based upon the evolving risk landscape. She may do this using a combination of computer-based training, live training, and gamification, but those techniques do not necessarily verify that the content is updated.</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>Alyssa ควรใช้การทบทวนเนื้อหาเป็นระยะ (periodic content reviews) เพื่อตรวจสอบอย่างต่อเนื่องว่าเนื้อหาในโปรแกรมของเธอนั้นตอบสนองต่อความต้องการขององค์กร และทันสมัยอยู่เสมอโดยอ้างอิงตามสภาวะความเสี่ยงที่เปลี่ยนแปลงไป (evolving risk landscape)
+เธออาจใช้เทคนิคต่างๆ ร่วมกันได้ เช่น การฝึกอบรมผ่านคอมพิวเตอร์, การอบรมแบบสด และการใช้เทคนิคเกม แต่เทคนิคเหล่านั้นไม่ได้ช่วยตรวจสอบหรือยืนยันว่าเนื้อหาได้รับการอัปเดตแล้วแต่อย่างใด</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr"/>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>1. Think Like a Manager / Fix the Process (คิดแบบผู้จัดการ เน้นที่กระบวนการ):
+     คนทำงานสายเทคนิคหรือคนทั่วไปมักจะมองหาเครื่องมือที่ฟังดูทันสมัย สะดุดตา (เช่น Gamification หรือ CBT) แต่ผู้จัดการความปลอดภัยที่ดีจะมองหา "กระบวนการควบคุมและตรวจสอบคุณภาพ" (Quality Assurance Process) ซึ่งในที่นี้คือการกำหนดตารางเวลาเพื่อ "ทบทวนเนื้อหา" (Content Reviews)
+2. Understand the Goal of Each Control (เข้าใจเป้าหมายที่แท้จริงของมาตรการ):
+     เป้าหมายของเทคนิคการสอน (A, B, D) มีไว้เพื่อเพิ่มการมีส่วนร่วม (Engagement) และการปรับเปลี่ยนพฤติกรรม (Behavior modification) ของพนักงาน
+     แต่เป้าหมายของ Content Reviews มีไว้เพื่อรับประกันความถูกต้อง ความสอดคล้อง และความสดใหม่ของข้อมูล (Information Integrity and Alignment)</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>security-awareness;governance</t>
+        </is>
+      </c>
+      <c r="X4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -803,6 +894,8 @@
       <c r="T5" s="3" t="n"/>
       <c r="U5" s="3" t="n"/>
       <c r="V5" s="3" t="n"/>
+      <c r="W5" s="3" t="n"/>
+      <c r="X5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -827,6 +920,8 @@
       <c r="T6" s="3" t="n"/>
       <c r="U6" s="3" t="n"/>
       <c r="V6" s="3" t="n"/>
+      <c r="W6" s="3" t="n"/>
+      <c r="X6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -851,6 +946,8 @@
       <c r="T7" s="3" t="n"/>
       <c r="U7" s="3" t="n"/>
       <c r="V7" s="3" t="n"/>
+      <c r="W7" s="3" t="n"/>
+      <c r="X7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -875,6 +972,8 @@
       <c r="T8" s="3" t="n"/>
       <c r="U8" s="3" t="n"/>
       <c r="V8" s="3" t="n"/>
+      <c r="W8" s="3" t="n"/>
+      <c r="X8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -899,6 +998,8 @@
       <c r="T9" s="3" t="n"/>
       <c r="U9" s="3" t="n"/>
       <c r="V9" s="3" t="n"/>
+      <c r="W9" s="3" t="n"/>
+      <c r="X9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -923,6 +1024,8 @@
       <c r="T10" s="3" t="n"/>
       <c r="U10" s="3" t="n"/>
       <c r="V10" s="3" t="n"/>
+      <c r="W10" s="3" t="n"/>
+      <c r="X10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -947,6 +1050,8 @@
       <c r="T11" s="3" t="n"/>
       <c r="U11" s="3" t="n"/>
       <c r="V11" s="3" t="n"/>
+      <c r="W11" s="3" t="n"/>
+      <c r="X11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -971,6 +1076,8 @@
       <c r="T12" s="3" t="n"/>
       <c r="U12" s="3" t="n"/>
       <c r="V12" s="3" t="n"/>
+      <c r="W12" s="3" t="n"/>
+      <c r="X12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -995,6 +1102,8 @@
       <c r="T13" s="3" t="n"/>
       <c r="U13" s="3" t="n"/>
       <c r="V13" s="3" t="n"/>
+      <c r="W13" s="3" t="n"/>
+      <c r="X13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -1019,6 +1128,8 @@
       <c r="T14" s="3" t="n"/>
       <c r="U14" s="3" t="n"/>
       <c r="V14" s="3" t="n"/>
+      <c r="W14" s="3" t="n"/>
+      <c r="X14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -1043,6 +1154,8 @@
       <c r="T15" s="3" t="n"/>
       <c r="U15" s="3" t="n"/>
       <c r="V15" s="3" t="n"/>
+      <c r="W15" s="3" t="n"/>
+      <c r="X15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -1067,6 +1180,8 @@
       <c r="T16" s="3" t="n"/>
       <c r="U16" s="3" t="n"/>
       <c r="V16" s="3" t="n"/>
+      <c r="W16" s="3" t="n"/>
+      <c r="X16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -1091,6 +1206,8 @@
       <c r="T17" s="3" t="n"/>
       <c r="U17" s="3" t="n"/>
       <c r="V17" s="3" t="n"/>
+      <c r="W17" s="3" t="n"/>
+      <c r="X17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -1115,6 +1232,8 @@
       <c r="T18" s="3" t="n"/>
       <c r="U18" s="3" t="n"/>
       <c r="V18" s="3" t="n"/>
+      <c r="W18" s="3" t="n"/>
+      <c r="X18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -1139,6 +1258,8 @@
       <c r="T19" s="3" t="n"/>
       <c r="U19" s="3" t="n"/>
       <c r="V19" s="3" t="n"/>
+      <c r="W19" s="3" t="n"/>
+      <c r="X19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -1163,6 +1284,8 @@
       <c r="T20" s="3" t="n"/>
       <c r="U20" s="3" t="n"/>
       <c r="V20" s="3" t="n"/>
+      <c r="W20" s="3" t="n"/>
+      <c r="X20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -1187,6 +1310,8 @@
       <c r="T21" s="3" t="n"/>
       <c r="U21" s="3" t="n"/>
       <c r="V21" s="3" t="n"/>
+      <c r="W21" s="3" t="n"/>
+      <c r="X21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -1211,6 +1336,8 @@
       <c r="T22" s="3" t="n"/>
       <c r="U22" s="3" t="n"/>
       <c r="V22" s="3" t="n"/>
+      <c r="W22" s="3" t="n"/>
+      <c r="X22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -1235,6 +1362,8 @@
       <c r="T23" s="3" t="n"/>
       <c r="U23" s="3" t="n"/>
       <c r="V23" s="3" t="n"/>
+      <c r="W23" s="3" t="n"/>
+      <c r="X23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -1259,6 +1388,8 @@
       <c r="T24" s="3" t="n"/>
       <c r="U24" s="3" t="n"/>
       <c r="V24" s="3" t="n"/>
+      <c r="W24" s="3" t="n"/>
+      <c r="X24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -1283,6 +1414,8 @@
       <c r="T25" s="3" t="n"/>
       <c r="U25" s="3" t="n"/>
       <c r="V25" s="3" t="n"/>
+      <c r="W25" s="3" t="n"/>
+      <c r="X25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -1307,6 +1440,8 @@
       <c r="T26" s="3" t="n"/>
       <c r="U26" s="3" t="n"/>
       <c r="V26" s="3" t="n"/>
+      <c r="W26" s="3" t="n"/>
+      <c r="X26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -1331,6 +1466,8 @@
       <c r="T27" s="3" t="n"/>
       <c r="U27" s="3" t="n"/>
       <c r="V27" s="3" t="n"/>
+      <c r="W27" s="3" t="n"/>
+      <c r="X27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -1355,6 +1492,8 @@
       <c r="T28" s="3" t="n"/>
       <c r="U28" s="3" t="n"/>
       <c r="V28" s="3" t="n"/>
+      <c r="W28" s="3" t="n"/>
+      <c r="X28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -1379,6 +1518,8 @@
       <c r="T29" s="3" t="n"/>
       <c r="U29" s="3" t="n"/>
       <c r="V29" s="3" t="n"/>
+      <c r="W29" s="3" t="n"/>
+      <c r="X29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -1403,6 +1544,8 @@
       <c r="T30" s="3" t="n"/>
       <c r="U30" s="3" t="n"/>
       <c r="V30" s="3" t="n"/>
+      <c r="W30" s="3" t="n"/>
+      <c r="X30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -1427,6 +1570,8 @@
       <c r="T31" s="3" t="n"/>
       <c r="U31" s="3" t="n"/>
       <c r="V31" s="3" t="n"/>
+      <c r="W31" s="3" t="n"/>
+      <c r="X31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -1451,6 +1596,8 @@
       <c r="T32" s="3" t="n"/>
       <c r="U32" s="3" t="n"/>
       <c r="V32" s="3" t="n"/>
+      <c r="W32" s="3" t="n"/>
+      <c r="X32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -1475,6 +1622,8 @@
       <c r="T33" s="3" t="n"/>
       <c r="U33" s="3" t="n"/>
       <c r="V33" s="3" t="n"/>
+      <c r="W33" s="3" t="n"/>
+      <c r="X33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -1499,6 +1648,8 @@
       <c r="T34" s="3" t="n"/>
       <c r="U34" s="3" t="n"/>
       <c r="V34" s="3" t="n"/>
+      <c r="W34" s="3" t="n"/>
+      <c r="X34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -1523,6 +1674,8 @@
       <c r="T35" s="3" t="n"/>
       <c r="U35" s="3" t="n"/>
       <c r="V35" s="3" t="n"/>
+      <c r="W35" s="3" t="n"/>
+      <c r="X35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -1547,6 +1700,8 @@
       <c r="T36" s="3" t="n"/>
       <c r="U36" s="3" t="n"/>
       <c r="V36" s="3" t="n"/>
+      <c r="W36" s="3" t="n"/>
+      <c r="X36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -1571,6 +1726,8 @@
       <c r="T37" s="3" t="n"/>
       <c r="U37" s="3" t="n"/>
       <c r="V37" s="3" t="n"/>
+      <c r="W37" s="3" t="n"/>
+      <c r="X37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -1595,6 +1752,8 @@
       <c r="T38" s="3" t="n"/>
       <c r="U38" s="3" t="n"/>
       <c r="V38" s="3" t="n"/>
+      <c r="W38" s="3" t="n"/>
+      <c r="X38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -1619,6 +1778,8 @@
       <c r="T39" s="3" t="n"/>
       <c r="U39" s="3" t="n"/>
       <c r="V39" s="3" t="n"/>
+      <c r="W39" s="3" t="n"/>
+      <c r="X39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -1643,6 +1804,8 @@
       <c r="T40" s="3" t="n"/>
       <c r="U40" s="3" t="n"/>
       <c r="V40" s="3" t="n"/>
+      <c r="W40" s="3" t="n"/>
+      <c r="X40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -1667,6 +1830,8 @@
       <c r="T41" s="3" t="n"/>
       <c r="U41" s="3" t="n"/>
       <c r="V41" s="3" t="n"/>
+      <c r="W41" s="3" t="n"/>
+      <c r="X41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -1691,6 +1856,8 @@
       <c r="T42" s="3" t="n"/>
       <c r="U42" s="3" t="n"/>
       <c r="V42" s="3" t="n"/>
+      <c r="W42" s="3" t="n"/>
+      <c r="X42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
@@ -1715,6 +1882,8 @@
       <c r="T43" s="3" t="n"/>
       <c r="U43" s="3" t="n"/>
       <c r="V43" s="3" t="n"/>
+      <c r="W43" s="3" t="n"/>
+      <c r="X43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -1739,6 +1908,8 @@
       <c r="T44" s="3" t="n"/>
       <c r="U44" s="3" t="n"/>
       <c r="V44" s="3" t="n"/>
+      <c r="W44" s="3" t="n"/>
+      <c r="X44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
@@ -1763,6 +1934,8 @@
       <c r="T45" s="3" t="n"/>
       <c r="U45" s="3" t="n"/>
       <c r="V45" s="3" t="n"/>
+      <c r="W45" s="3" t="n"/>
+      <c r="X45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -1787,6 +1960,8 @@
       <c r="T46" s="3" t="n"/>
       <c r="U46" s="3" t="n"/>
       <c r="V46" s="3" t="n"/>
+      <c r="W46" s="3" t="n"/>
+      <c r="X46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
@@ -1811,6 +1986,8 @@
       <c r="T47" s="3" t="n"/>
       <c r="U47" s="3" t="n"/>
       <c r="V47" s="3" t="n"/>
+      <c r="W47" s="3" t="n"/>
+      <c r="X47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -1835,6 +2012,8 @@
       <c r="T48" s="3" t="n"/>
       <c r="U48" s="3" t="n"/>
       <c r="V48" s="3" t="n"/>
+      <c r="W48" s="3" t="n"/>
+      <c r="X48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
@@ -1859,6 +2038,8 @@
       <c r="T49" s="3" t="n"/>
       <c r="U49" s="3" t="n"/>
       <c r="V49" s="3" t="n"/>
+      <c r="W49" s="3" t="n"/>
+      <c r="X49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -1883,6 +2064,8 @@
       <c r="T50" s="3" t="n"/>
       <c r="U50" s="3" t="n"/>
       <c r="V50" s="3" t="n"/>
+      <c r="W50" s="3" t="n"/>
+      <c r="X50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
@@ -1907,6 +2090,8 @@
       <c r="T51" s="3" t="n"/>
       <c r="U51" s="3" t="n"/>
       <c r="V51" s="3" t="n"/>
+      <c r="W51" s="3" t="n"/>
+      <c r="X51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -1931,6 +2116,8 @@
       <c r="T52" s="3" t="n"/>
       <c r="U52" s="3" t="n"/>
       <c r="V52" s="3" t="n"/>
+      <c r="W52" s="3" t="n"/>
+      <c r="X52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
@@ -1955,6 +2142,8 @@
       <c r="T53" s="3" t="n"/>
       <c r="U53" s="3" t="n"/>
       <c r="V53" s="3" t="n"/>
+      <c r="W53" s="3" t="n"/>
+      <c r="X53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -1979,6 +2168,8 @@
       <c r="T54" s="3" t="n"/>
       <c r="U54" s="3" t="n"/>
       <c r="V54" s="3" t="n"/>
+      <c r="W54" s="3" t="n"/>
+      <c r="X54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
@@ -2003,6 +2194,8 @@
       <c r="T55" s="3" t="n"/>
       <c r="U55" s="3" t="n"/>
       <c r="V55" s="3" t="n"/>
+      <c r="W55" s="3" t="n"/>
+      <c r="X55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -2027,6 +2220,8 @@
       <c r="T56" s="3" t="n"/>
       <c r="U56" s="3" t="n"/>
       <c r="V56" s="3" t="n"/>
+      <c r="W56" s="3" t="n"/>
+      <c r="X56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
@@ -2051,6 +2246,8 @@
       <c r="T57" s="3" t="n"/>
       <c r="U57" s="3" t="n"/>
       <c r="V57" s="3" t="n"/>
+      <c r="W57" s="3" t="n"/>
+      <c r="X57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -2075,6 +2272,8 @@
       <c r="T58" s="3" t="n"/>
       <c r="U58" s="3" t="n"/>
       <c r="V58" s="3" t="n"/>
+      <c r="W58" s="3" t="n"/>
+      <c r="X58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
@@ -2099,6 +2298,8 @@
       <c r="T59" s="3" t="n"/>
       <c r="U59" s="3" t="n"/>
       <c r="V59" s="3" t="n"/>
+      <c r="W59" s="3" t="n"/>
+      <c r="X59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -2123,6 +2324,8 @@
       <c r="T60" s="3" t="n"/>
       <c r="U60" s="3" t="n"/>
       <c r="V60" s="3" t="n"/>
+      <c r="W60" s="3" t="n"/>
+      <c r="X60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
@@ -2147,6 +2350,8 @@
       <c r="T61" s="3" t="n"/>
       <c r="U61" s="3" t="n"/>
       <c r="V61" s="3" t="n"/>
+      <c r="W61" s="3" t="n"/>
+      <c r="X61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -2171,6 +2376,8 @@
       <c r="T62" s="3" t="n"/>
       <c r="U62" s="3" t="n"/>
       <c r="V62" s="3" t="n"/>
+      <c r="W62" s="3" t="n"/>
+      <c r="X62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n"/>
@@ -2195,6 +2402,8 @@
       <c r="T63" s="3" t="n"/>
       <c r="U63" s="3" t="n"/>
       <c r="V63" s="3" t="n"/>
+      <c r="W63" s="3" t="n"/>
+      <c r="X63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -2219,6 +2428,8 @@
       <c r="T64" s="3" t="n"/>
       <c r="U64" s="3" t="n"/>
       <c r="V64" s="3" t="n"/>
+      <c r="W64" s="3" t="n"/>
+      <c r="X64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
@@ -2243,6 +2454,8 @@
       <c r="T65" s="3" t="n"/>
       <c r="U65" s="3" t="n"/>
       <c r="V65" s="3" t="n"/>
+      <c r="W65" s="3" t="n"/>
+      <c r="X65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -2267,6 +2480,8 @@
       <c r="T66" s="3" t="n"/>
       <c r="U66" s="3" t="n"/>
       <c r="V66" s="3" t="n"/>
+      <c r="W66" s="3" t="n"/>
+      <c r="X66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
@@ -2291,6 +2506,8 @@
       <c r="T67" s="3" t="n"/>
       <c r="U67" s="3" t="n"/>
       <c r="V67" s="3" t="n"/>
+      <c r="W67" s="3" t="n"/>
+      <c r="X67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -2315,6 +2532,8 @@
       <c r="T68" s="3" t="n"/>
       <c r="U68" s="3" t="n"/>
       <c r="V68" s="3" t="n"/>
+      <c r="W68" s="3" t="n"/>
+      <c r="X68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n"/>
@@ -2339,6 +2558,8 @@
       <c r="T69" s="3" t="n"/>
       <c r="U69" s="3" t="n"/>
       <c r="V69" s="3" t="n"/>
+      <c r="W69" s="3" t="n"/>
+      <c r="X69" s="3" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
@@ -2363,6 +2584,8 @@
       <c r="T70" s="3" t="n"/>
       <c r="U70" s="3" t="n"/>
       <c r="V70" s="3" t="n"/>
+      <c r="W70" s="3" t="n"/>
+      <c r="X70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n"/>
@@ -2387,6 +2610,8 @@
       <c r="T71" s="3" t="n"/>
       <c r="U71" s="3" t="n"/>
       <c r="V71" s="3" t="n"/>
+      <c r="W71" s="3" t="n"/>
+      <c r="X71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
@@ -2411,6 +2636,8 @@
       <c r="T72" s="3" t="n"/>
       <c r="U72" s="3" t="n"/>
       <c r="V72" s="3" t="n"/>
+      <c r="W72" s="3" t="n"/>
+      <c r="X72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n"/>
@@ -2435,6 +2662,8 @@
       <c r="T73" s="3" t="n"/>
       <c r="U73" s="3" t="n"/>
       <c r="V73" s="3" t="n"/>
+      <c r="W73" s="3" t="n"/>
+      <c r="X73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
@@ -2459,6 +2688,8 @@
       <c r="T74" s="3" t="n"/>
       <c r="U74" s="3" t="n"/>
       <c r="V74" s="3" t="n"/>
+      <c r="W74" s="3" t="n"/>
+      <c r="X74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n"/>
@@ -2483,6 +2714,8 @@
       <c r="T75" s="3" t="n"/>
       <c r="U75" s="3" t="n"/>
       <c r="V75" s="3" t="n"/>
+      <c r="W75" s="3" t="n"/>
+      <c r="X75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
@@ -2507,6 +2740,8 @@
       <c r="T76" s="3" t="n"/>
       <c r="U76" s="3" t="n"/>
       <c r="V76" s="3" t="n"/>
+      <c r="W76" s="3" t="n"/>
+      <c r="X76" s="3" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n"/>
@@ -2531,6 +2766,8 @@
       <c r="T77" s="3" t="n"/>
       <c r="U77" s="3" t="n"/>
       <c r="V77" s="3" t="n"/>
+      <c r="W77" s="3" t="n"/>
+      <c r="X77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
@@ -2555,6 +2792,8 @@
       <c r="T78" s="3" t="n"/>
       <c r="U78" s="3" t="n"/>
       <c r="V78" s="3" t="n"/>
+      <c r="W78" s="3" t="n"/>
+      <c r="X78" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n"/>
@@ -2579,6 +2818,8 @@
       <c r="T79" s="3" t="n"/>
       <c r="U79" s="3" t="n"/>
       <c r="V79" s="3" t="n"/>
+      <c r="W79" s="3" t="n"/>
+      <c r="X79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
@@ -2603,6 +2844,8 @@
       <c r="T80" s="3" t="n"/>
       <c r="U80" s="3" t="n"/>
       <c r="V80" s="3" t="n"/>
+      <c r="W80" s="3" t="n"/>
+      <c r="X80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n"/>
@@ -2627,6 +2870,8 @@
       <c r="T81" s="3" t="n"/>
       <c r="U81" s="3" t="n"/>
       <c r="V81" s="3" t="n"/>
+      <c r="W81" s="3" t="n"/>
+      <c r="X81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
@@ -2651,6 +2896,8 @@
       <c r="T82" s="3" t="n"/>
       <c r="U82" s="3" t="n"/>
       <c r="V82" s="3" t="n"/>
+      <c r="W82" s="3" t="n"/>
+      <c r="X82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n"/>
@@ -2675,6 +2922,8 @@
       <c r="T83" s="3" t="n"/>
       <c r="U83" s="3" t="n"/>
       <c r="V83" s="3" t="n"/>
+      <c r="W83" s="3" t="n"/>
+      <c r="X83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n"/>
@@ -2699,6 +2948,8 @@
       <c r="T84" s="3" t="n"/>
       <c r="U84" s="3" t="n"/>
       <c r="V84" s="3" t="n"/>
+      <c r="W84" s="3" t="n"/>
+      <c r="X84" s="3" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n"/>
@@ -2723,6 +2974,8 @@
       <c r="T85" s="3" t="n"/>
       <c r="U85" s="3" t="n"/>
       <c r="V85" s="3" t="n"/>
+      <c r="W85" s="3" t="n"/>
+      <c r="X85" s="3" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n"/>
@@ -2747,6 +3000,8 @@
       <c r="T86" s="3" t="n"/>
       <c r="U86" s="3" t="n"/>
       <c r="V86" s="3" t="n"/>
+      <c r="W86" s="3" t="n"/>
+      <c r="X86" s="3" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n"/>
@@ -2771,6 +3026,8 @@
       <c r="T87" s="3" t="n"/>
       <c r="U87" s="3" t="n"/>
       <c r="V87" s="3" t="n"/>
+      <c r="W87" s="3" t="n"/>
+      <c r="X87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n"/>
@@ -2795,6 +3052,8 @@
       <c r="T88" s="3" t="n"/>
       <c r="U88" s="3" t="n"/>
       <c r="V88" s="3" t="n"/>
+      <c r="W88" s="3" t="n"/>
+      <c r="X88" s="3" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n"/>
@@ -2819,6 +3078,8 @@
       <c r="T89" s="3" t="n"/>
       <c r="U89" s="3" t="n"/>
       <c r="V89" s="3" t="n"/>
+      <c r="W89" s="3" t="n"/>
+      <c r="X89" s="3" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n"/>
@@ -2843,6 +3104,8 @@
       <c r="T90" s="3" t="n"/>
       <c r="U90" s="3" t="n"/>
       <c r="V90" s="3" t="n"/>
+      <c r="W90" s="3" t="n"/>
+      <c r="X90" s="3" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n"/>
@@ -2867,6 +3130,8 @@
       <c r="T91" s="3" t="n"/>
       <c r="U91" s="3" t="n"/>
       <c r="V91" s="3" t="n"/>
+      <c r="W91" s="3" t="n"/>
+      <c r="X91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n"/>
@@ -2891,6 +3156,8 @@
       <c r="T92" s="3" t="n"/>
       <c r="U92" s="3" t="n"/>
       <c r="V92" s="3" t="n"/>
+      <c r="W92" s="3" t="n"/>
+      <c r="X92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n"/>
@@ -2915,6 +3182,8 @@
       <c r="T93" s="3" t="n"/>
       <c r="U93" s="3" t="n"/>
       <c r="V93" s="3" t="n"/>
+      <c r="W93" s="3" t="n"/>
+      <c r="X93" s="3" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n"/>
@@ -2939,6 +3208,8 @@
       <c r="T94" s="3" t="n"/>
       <c r="U94" s="3" t="n"/>
       <c r="V94" s="3" t="n"/>
+      <c r="W94" s="3" t="n"/>
+      <c r="X94" s="3" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n"/>
@@ -2963,6 +3234,8 @@
       <c r="T95" s="3" t="n"/>
       <c r="U95" s="3" t="n"/>
       <c r="V95" s="3" t="n"/>
+      <c r="W95" s="3" t="n"/>
+      <c r="X95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n"/>
@@ -2987,6 +3260,8 @@
       <c r="T96" s="3" t="n"/>
       <c r="U96" s="3" t="n"/>
       <c r="V96" s="3" t="n"/>
+      <c r="W96" s="3" t="n"/>
+      <c r="X96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n"/>
@@ -3011,6 +3286,8 @@
       <c r="T97" s="3" t="n"/>
       <c r="U97" s="3" t="n"/>
       <c r="V97" s="3" t="n"/>
+      <c r="W97" s="3" t="n"/>
+      <c r="X97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n"/>
@@ -3035,6 +3312,8 @@
       <c r="T98" s="3" t="n"/>
       <c r="U98" s="3" t="n"/>
       <c r="V98" s="3" t="n"/>
+      <c r="W98" s="3" t="n"/>
+      <c r="X98" s="3" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n"/>
@@ -3059,6 +3338,8 @@
       <c r="T99" s="3" t="n"/>
       <c r="U99" s="3" t="n"/>
       <c r="V99" s="3" t="n"/>
+      <c r="W99" s="3" t="n"/>
+      <c r="X99" s="3" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n"/>
@@ -3083,6 +3364,8 @@
       <c r="T100" s="3" t="n"/>
       <c r="U100" s="3" t="n"/>
       <c r="V100" s="3" t="n"/>
+      <c r="W100" s="3" t="n"/>
+      <c r="X100" s="3" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n"/>
@@ -3107,6 +3390,8 @@
       <c r="T101" s="3" t="n"/>
       <c r="U101" s="3" t="n"/>
       <c r="V101" s="3" t="n"/>
+      <c r="W101" s="3" t="n"/>
+      <c r="X101" s="3" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n"/>
@@ -3131,6 +3416,8 @@
       <c r="T102" s="3" t="n"/>
       <c r="U102" s="3" t="n"/>
       <c r="V102" s="3" t="n"/>
+      <c r="W102" s="3" t="n"/>
+      <c r="X102" s="3" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n"/>
@@ -3155,6 +3442,8 @@
       <c r="T103" s="3" t="n"/>
       <c r="U103" s="3" t="n"/>
       <c r="V103" s="3" t="n"/>
+      <c r="W103" s="3" t="n"/>
+      <c r="X103" s="3" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n"/>
@@ -3179,6 +3468,8 @@
       <c r="T104" s="3" t="n"/>
       <c r="U104" s="3" t="n"/>
       <c r="V104" s="3" t="n"/>
+      <c r="W104" s="3" t="n"/>
+      <c r="X104" s="3" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n"/>
@@ -3203,6 +3494,8 @@
       <c r="T105" s="3" t="n"/>
       <c r="U105" s="3" t="n"/>
       <c r="V105" s="3" t="n"/>
+      <c r="W105" s="3" t="n"/>
+      <c r="X105" s="3" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n"/>
@@ -3227,6 +3520,8 @@
       <c r="T106" s="3" t="n"/>
       <c r="U106" s="3" t="n"/>
       <c r="V106" s="3" t="n"/>
+      <c r="W106" s="3" t="n"/>
+      <c r="X106" s="3" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n"/>
@@ -3251,6 +3546,8 @@
       <c r="T107" s="3" t="n"/>
       <c r="U107" s="3" t="n"/>
       <c r="V107" s="3" t="n"/>
+      <c r="W107" s="3" t="n"/>
+      <c r="X107" s="3" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n"/>
@@ -3275,6 +3572,8 @@
       <c r="T108" s="3" t="n"/>
       <c r="U108" s="3" t="n"/>
       <c r="V108" s="3" t="n"/>
+      <c r="W108" s="3" t="n"/>
+      <c r="X108" s="3" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n"/>
@@ -3299,6 +3598,8 @@
       <c r="T109" s="3" t="n"/>
       <c r="U109" s="3" t="n"/>
       <c r="V109" s="3" t="n"/>
+      <c r="W109" s="3" t="n"/>
+      <c r="X109" s="3" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n"/>
@@ -3323,6 +3624,8 @@
       <c r="T110" s="3" t="n"/>
       <c r="U110" s="3" t="n"/>
       <c r="V110" s="3" t="n"/>
+      <c r="W110" s="3" t="n"/>
+      <c r="X110" s="3" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="3" t="n"/>
@@ -3347,6 +3650,8 @@
       <c r="T111" s="3" t="n"/>
       <c r="U111" s="3" t="n"/>
       <c r="V111" s="3" t="n"/>
+      <c r="W111" s="3" t="n"/>
+      <c r="X111" s="3" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="3" t="n"/>
@@ -3371,6 +3676,8 @@
       <c r="T112" s="3" t="n"/>
       <c r="U112" s="3" t="n"/>
       <c r="V112" s="3" t="n"/>
+      <c r="W112" s="3" t="n"/>
+      <c r="X112" s="3" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n"/>
@@ -3395,6 +3702,8 @@
       <c r="T113" s="3" t="n"/>
       <c r="U113" s="3" t="n"/>
       <c r="V113" s="3" t="n"/>
+      <c r="W113" s="3" t="n"/>
+      <c r="X113" s="3" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="n"/>
@@ -3419,6 +3728,8 @@
       <c r="T114" s="3" t="n"/>
       <c r="U114" s="3" t="n"/>
       <c r="V114" s="3" t="n"/>
+      <c r="W114" s="3" t="n"/>
+      <c r="X114" s="3" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="n"/>
@@ -3443,6 +3754,8 @@
       <c r="T115" s="3" t="n"/>
       <c r="U115" s="3" t="n"/>
       <c r="V115" s="3" t="n"/>
+      <c r="W115" s="3" t="n"/>
+      <c r="X115" s="3" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="3" t="n"/>
@@ -3467,6 +3780,8 @@
       <c r="T116" s="3" t="n"/>
       <c r="U116" s="3" t="n"/>
       <c r="V116" s="3" t="n"/>
+      <c r="W116" s="3" t="n"/>
+      <c r="X116" s="3" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="3" t="n"/>
@@ -3491,6 +3806,8 @@
       <c r="T117" s="3" t="n"/>
       <c r="U117" s="3" t="n"/>
       <c r="V117" s="3" t="n"/>
+      <c r="W117" s="3" t="n"/>
+      <c r="X117" s="3" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="3" t="n"/>
@@ -3515,6 +3832,8 @@
       <c r="T118" s="3" t="n"/>
       <c r="U118" s="3" t="n"/>
       <c r="V118" s="3" t="n"/>
+      <c r="W118" s="3" t="n"/>
+      <c r="X118" s="3" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="3" t="n"/>
@@ -3539,6 +3858,8 @@
       <c r="T119" s="3" t="n"/>
       <c r="U119" s="3" t="n"/>
       <c r="V119" s="3" t="n"/>
+      <c r="W119" s="3" t="n"/>
+      <c r="X119" s="3" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="3" t="n"/>
@@ -3563,6 +3884,8 @@
       <c r="T120" s="3" t="n"/>
       <c r="U120" s="3" t="n"/>
       <c r="V120" s="3" t="n"/>
+      <c r="W120" s="3" t="n"/>
+      <c r="X120" s="3" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="3" t="n"/>
@@ -3587,6 +3910,8 @@
       <c r="T121" s="3" t="n"/>
       <c r="U121" s="3" t="n"/>
       <c r="V121" s="3" t="n"/>
+      <c r="W121" s="3" t="n"/>
+      <c r="X121" s="3" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="3" t="n"/>
@@ -3611,6 +3936,8 @@
       <c r="T122" s="3" t="n"/>
       <c r="U122" s="3" t="n"/>
       <c r="V122" s="3" t="n"/>
+      <c r="W122" s="3" t="n"/>
+      <c r="X122" s="3" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="3" t="n"/>
@@ -3635,6 +3962,8 @@
       <c r="T123" s="3" t="n"/>
       <c r="U123" s="3" t="n"/>
       <c r="V123" s="3" t="n"/>
+      <c r="W123" s="3" t="n"/>
+      <c r="X123" s="3" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="3" t="n"/>
@@ -3659,6 +3988,8 @@
       <c r="T124" s="3" t="n"/>
       <c r="U124" s="3" t="n"/>
       <c r="V124" s="3" t="n"/>
+      <c r="W124" s="3" t="n"/>
+      <c r="X124" s="3" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="3" t="n"/>
@@ -3683,6 +4014,8 @@
       <c r="T125" s="3" t="n"/>
       <c r="U125" s="3" t="n"/>
       <c r="V125" s="3" t="n"/>
+      <c r="W125" s="3" t="n"/>
+      <c r="X125" s="3" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="3" t="n"/>
@@ -3707,6 +4040,8 @@
       <c r="T126" s="3" t="n"/>
       <c r="U126" s="3" t="n"/>
       <c r="V126" s="3" t="n"/>
+      <c r="W126" s="3" t="n"/>
+      <c r="X126" s="3" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="3" t="n"/>
@@ -3731,6 +4066,8 @@
       <c r="T127" s="3" t="n"/>
       <c r="U127" s="3" t="n"/>
       <c r="V127" s="3" t="n"/>
+      <c r="W127" s="3" t="n"/>
+      <c r="X127" s="3" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="3" t="n"/>
@@ -3755,6 +4092,8 @@
       <c r="T128" s="3" t="n"/>
       <c r="U128" s="3" t="n"/>
       <c r="V128" s="3" t="n"/>
+      <c r="W128" s="3" t="n"/>
+      <c r="X128" s="3" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="3" t="n"/>
@@ -3779,6 +4118,8 @@
       <c r="T129" s="3" t="n"/>
       <c r="U129" s="3" t="n"/>
       <c r="V129" s="3" t="n"/>
+      <c r="W129" s="3" t="n"/>
+      <c r="X129" s="3" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="3" t="n"/>
@@ -3803,6 +4144,8 @@
       <c r="T130" s="3" t="n"/>
       <c r="U130" s="3" t="n"/>
       <c r="V130" s="3" t="n"/>
+      <c r="W130" s="3" t="n"/>
+      <c r="X130" s="3" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="3" t="n"/>
@@ -3827,6 +4170,8 @@
       <c r="T131" s="3" t="n"/>
       <c r="U131" s="3" t="n"/>
       <c r="V131" s="3" t="n"/>
+      <c r="W131" s="3" t="n"/>
+      <c r="X131" s="3" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="3" t="n"/>
@@ -3851,6 +4196,8 @@
       <c r="T132" s="3" t="n"/>
       <c r="U132" s="3" t="n"/>
       <c r="V132" s="3" t="n"/>
+      <c r="W132" s="3" t="n"/>
+      <c r="X132" s="3" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="3" t="n"/>
@@ -3875,6 +4222,8 @@
       <c r="T133" s="3" t="n"/>
       <c r="U133" s="3" t="n"/>
       <c r="V133" s="3" t="n"/>
+      <c r="W133" s="3" t="n"/>
+      <c r="X133" s="3" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="3" t="n"/>
@@ -3899,6 +4248,8 @@
       <c r="T134" s="3" t="n"/>
       <c r="U134" s="3" t="n"/>
       <c r="V134" s="3" t="n"/>
+      <c r="W134" s="3" t="n"/>
+      <c r="X134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="3" t="n"/>
@@ -3923,6 +4274,8 @@
       <c r="T135" s="3" t="n"/>
       <c r="U135" s="3" t="n"/>
       <c r="V135" s="3" t="n"/>
+      <c r="W135" s="3" t="n"/>
+      <c r="X135" s="3" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="3" t="n"/>
@@ -3947,6 +4300,8 @@
       <c r="T136" s="3" t="n"/>
       <c r="U136" s="3" t="n"/>
       <c r="V136" s="3" t="n"/>
+      <c r="W136" s="3" t="n"/>
+      <c r="X136" s="3" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="3" t="n"/>
@@ -3971,6 +4326,8 @@
       <c r="T137" s="3" t="n"/>
       <c r="U137" s="3" t="n"/>
       <c r="V137" s="3" t="n"/>
+      <c r="W137" s="3" t="n"/>
+      <c r="X137" s="3" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="3" t="n"/>
@@ -3995,6 +4352,8 @@
       <c r="T138" s="3" t="n"/>
       <c r="U138" s="3" t="n"/>
       <c r="V138" s="3" t="n"/>
+      <c r="W138" s="3" t="n"/>
+      <c r="X138" s="3" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="3" t="n"/>
@@ -4019,6 +4378,8 @@
       <c r="T139" s="3" t="n"/>
       <c r="U139" s="3" t="n"/>
       <c r="V139" s="3" t="n"/>
+      <c r="W139" s="3" t="n"/>
+      <c r="X139" s="3" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="3" t="n"/>
@@ -4043,6 +4404,8 @@
       <c r="T140" s="3" t="n"/>
       <c r="U140" s="3" t="n"/>
       <c r="V140" s="3" t="n"/>
+      <c r="W140" s="3" t="n"/>
+      <c r="X140" s="3" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="3" t="n"/>
@@ -4067,6 +4430,8 @@
       <c r="T141" s="3" t="n"/>
       <c r="U141" s="3" t="n"/>
       <c r="V141" s="3" t="n"/>
+      <c r="W141" s="3" t="n"/>
+      <c r="X141" s="3" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="3" t="n"/>
@@ -4091,6 +4456,8 @@
       <c r="T142" s="3" t="n"/>
       <c r="U142" s="3" t="n"/>
       <c r="V142" s="3" t="n"/>
+      <c r="W142" s="3" t="n"/>
+      <c r="X142" s="3" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="3" t="n"/>
@@ -4115,6 +4482,8 @@
       <c r="T143" s="3" t="n"/>
       <c r="U143" s="3" t="n"/>
       <c r="V143" s="3" t="n"/>
+      <c r="W143" s="3" t="n"/>
+      <c r="X143" s="3" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="3" t="n"/>
@@ -4139,6 +4508,8 @@
       <c r="T144" s="3" t="n"/>
       <c r="U144" s="3" t="n"/>
       <c r="V144" s="3" t="n"/>
+      <c r="W144" s="3" t="n"/>
+      <c r="X144" s="3" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="3" t="n"/>
@@ -4163,6 +4534,8 @@
       <c r="T145" s="3" t="n"/>
       <c r="U145" s="3" t="n"/>
       <c r="V145" s="3" t="n"/>
+      <c r="W145" s="3" t="n"/>
+      <c r="X145" s="3" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="3" t="n"/>
@@ -4187,6 +4560,8 @@
       <c r="T146" s="3" t="n"/>
       <c r="U146" s="3" t="n"/>
       <c r="V146" s="3" t="n"/>
+      <c r="W146" s="3" t="n"/>
+      <c r="X146" s="3" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="3" t="n"/>
@@ -4211,6 +4586,8 @@
       <c r="T147" s="3" t="n"/>
       <c r="U147" s="3" t="n"/>
       <c r="V147" s="3" t="n"/>
+      <c r="W147" s="3" t="n"/>
+      <c r="X147" s="3" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="3" t="n"/>
@@ -4235,6 +4612,8 @@
       <c r="T148" s="3" t="n"/>
       <c r="U148" s="3" t="n"/>
       <c r="V148" s="3" t="n"/>
+      <c r="W148" s="3" t="n"/>
+      <c r="X148" s="3" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="3" t="n"/>
@@ -4259,6 +4638,8 @@
       <c r="T149" s="3" t="n"/>
       <c r="U149" s="3" t="n"/>
       <c r="V149" s="3" t="n"/>
+      <c r="W149" s="3" t="n"/>
+      <c r="X149" s="3" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="3" t="n"/>
@@ -4283,6 +4664,8 @@
       <c r="T150" s="3" t="n"/>
       <c r="U150" s="3" t="n"/>
       <c r="V150" s="3" t="n"/>
+      <c r="W150" s="3" t="n"/>
+      <c r="X150" s="3" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="3" t="n"/>
@@ -4307,6 +4690,8 @@
       <c r="T151" s="3" t="n"/>
       <c r="U151" s="3" t="n"/>
       <c r="V151" s="3" t="n"/>
+      <c r="W151" s="3" t="n"/>
+      <c r="X151" s="3" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="3" t="n"/>
@@ -4331,6 +4716,8 @@
       <c r="T152" s="3" t="n"/>
       <c r="U152" s="3" t="n"/>
       <c r="V152" s="3" t="n"/>
+      <c r="W152" s="3" t="n"/>
+      <c r="X152" s="3" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="3" t="n"/>
@@ -4355,6 +4742,8 @@
       <c r="T153" s="3" t="n"/>
       <c r="U153" s="3" t="n"/>
       <c r="V153" s="3" t="n"/>
+      <c r="W153" s="3" t="n"/>
+      <c r="X153" s="3" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="3" t="n"/>
@@ -4379,6 +4768,8 @@
       <c r="T154" s="3" t="n"/>
       <c r="U154" s="3" t="n"/>
       <c r="V154" s="3" t="n"/>
+      <c r="W154" s="3" t="n"/>
+      <c r="X154" s="3" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="3" t="n"/>
@@ -4403,6 +4794,8 @@
       <c r="T155" s="3" t="n"/>
       <c r="U155" s="3" t="n"/>
       <c r="V155" s="3" t="n"/>
+      <c r="W155" s="3" t="n"/>
+      <c r="X155" s="3" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="3" t="n"/>
@@ -4427,6 +4820,8 @@
       <c r="T156" s="3" t="n"/>
       <c r="U156" s="3" t="n"/>
       <c r="V156" s="3" t="n"/>
+      <c r="W156" s="3" t="n"/>
+      <c r="X156" s="3" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="3" t="n"/>
@@ -4451,6 +4846,8 @@
       <c r="T157" s="3" t="n"/>
       <c r="U157" s="3" t="n"/>
       <c r="V157" s="3" t="n"/>
+      <c r="W157" s="3" t="n"/>
+      <c r="X157" s="3" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="3" t="n"/>
@@ -4475,6 +4872,8 @@
       <c r="T158" s="3" t="n"/>
       <c r="U158" s="3" t="n"/>
       <c r="V158" s="3" t="n"/>
+      <c r="W158" s="3" t="n"/>
+      <c r="X158" s="3" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="3" t="n"/>
@@ -4499,6 +4898,8 @@
       <c r="T159" s="3" t="n"/>
       <c r="U159" s="3" t="n"/>
       <c r="V159" s="3" t="n"/>
+      <c r="W159" s="3" t="n"/>
+      <c r="X159" s="3" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="3" t="n"/>
@@ -4523,6 +4924,8 @@
       <c r="T160" s="3" t="n"/>
       <c r="U160" s="3" t="n"/>
       <c r="V160" s="3" t="n"/>
+      <c r="W160" s="3" t="n"/>
+      <c r="X160" s="3" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="3" t="n"/>
@@ -4547,6 +4950,8 @@
       <c r="T161" s="3" t="n"/>
       <c r="U161" s="3" t="n"/>
       <c r="V161" s="3" t="n"/>
+      <c r="W161" s="3" t="n"/>
+      <c r="X161" s="3" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="3" t="n"/>
@@ -4571,6 +4976,8 @@
       <c r="T162" s="3" t="n"/>
       <c r="U162" s="3" t="n"/>
       <c r="V162" s="3" t="n"/>
+      <c r="W162" s="3" t="n"/>
+      <c r="X162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="3" t="n"/>
@@ -4595,6 +5002,8 @@
       <c r="T163" s="3" t="n"/>
       <c r="U163" s="3" t="n"/>
       <c r="V163" s="3" t="n"/>
+      <c r="W163" s="3" t="n"/>
+      <c r="X163" s="3" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="3" t="n"/>
@@ -4619,6 +5028,8 @@
       <c r="T164" s="3" t="n"/>
       <c r="U164" s="3" t="n"/>
       <c r="V164" s="3" t="n"/>
+      <c r="W164" s="3" t="n"/>
+      <c r="X164" s="3" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="3" t="n"/>
@@ -4643,6 +5054,8 @@
       <c r="T165" s="3" t="n"/>
       <c r="U165" s="3" t="n"/>
       <c r="V165" s="3" t="n"/>
+      <c r="W165" s="3" t="n"/>
+      <c r="X165" s="3" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="3" t="n"/>
@@ -4667,6 +5080,8 @@
       <c r="T166" s="3" t="n"/>
       <c r="U166" s="3" t="n"/>
       <c r="V166" s="3" t="n"/>
+      <c r="W166" s="3" t="n"/>
+      <c r="X166" s="3" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="3" t="n"/>
@@ -4691,6 +5106,8 @@
       <c r="T167" s="3" t="n"/>
       <c r="U167" s="3" t="n"/>
       <c r="V167" s="3" t="n"/>
+      <c r="W167" s="3" t="n"/>
+      <c r="X167" s="3" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="3" t="n"/>
@@ -4715,6 +5132,8 @@
       <c r="T168" s="3" t="n"/>
       <c r="U168" s="3" t="n"/>
       <c r="V168" s="3" t="n"/>
+      <c r="W168" s="3" t="n"/>
+      <c r="X168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="3" t="n"/>
@@ -4739,6 +5158,8 @@
       <c r="T169" s="3" t="n"/>
       <c r="U169" s="3" t="n"/>
       <c r="V169" s="3" t="n"/>
+      <c r="W169" s="3" t="n"/>
+      <c r="X169" s="3" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="3" t="n"/>
@@ -4763,6 +5184,8 @@
       <c r="T170" s="3" t="n"/>
       <c r="U170" s="3" t="n"/>
       <c r="V170" s="3" t="n"/>
+      <c r="W170" s="3" t="n"/>
+      <c r="X170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="3" t="n"/>
@@ -4787,6 +5210,8 @@
       <c r="T171" s="3" t="n"/>
       <c r="U171" s="3" t="n"/>
       <c r="V171" s="3" t="n"/>
+      <c r="W171" s="3" t="n"/>
+      <c r="X171" s="3" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="3" t="n"/>
@@ -4811,6 +5236,8 @@
       <c r="T172" s="3" t="n"/>
       <c r="U172" s="3" t="n"/>
       <c r="V172" s="3" t="n"/>
+      <c r="W172" s="3" t="n"/>
+      <c r="X172" s="3" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="3" t="n"/>
@@ -4835,6 +5262,8 @@
       <c r="T173" s="3" t="n"/>
       <c r="U173" s="3" t="n"/>
       <c r="V173" s="3" t="n"/>
+      <c r="W173" s="3" t="n"/>
+      <c r="X173" s="3" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="3" t="n"/>
@@ -4859,6 +5288,8 @@
       <c r="T174" s="3" t="n"/>
       <c r="U174" s="3" t="n"/>
       <c r="V174" s="3" t="n"/>
+      <c r="W174" s="3" t="n"/>
+      <c r="X174" s="3" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="3" t="n"/>
@@ -4883,6 +5314,8 @@
       <c r="T175" s="3" t="n"/>
       <c r="U175" s="3" t="n"/>
       <c r="V175" s="3" t="n"/>
+      <c r="W175" s="3" t="n"/>
+      <c r="X175" s="3" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="3" t="n"/>
@@ -4907,6 +5340,8 @@
       <c r="T176" s="3" t="n"/>
       <c r="U176" s="3" t="n"/>
       <c r="V176" s="3" t="n"/>
+      <c r="W176" s="3" t="n"/>
+      <c r="X176" s="3" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="3" t="n"/>
@@ -4931,6 +5366,8 @@
       <c r="T177" s="3" t="n"/>
       <c r="U177" s="3" t="n"/>
       <c r="V177" s="3" t="n"/>
+      <c r="W177" s="3" t="n"/>
+      <c r="X177" s="3" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="3" t="n"/>
@@ -4955,6 +5392,8 @@
       <c r="T178" s="3" t="n"/>
       <c r="U178" s="3" t="n"/>
       <c r="V178" s="3" t="n"/>
+      <c r="W178" s="3" t="n"/>
+      <c r="X178" s="3" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="3" t="n"/>
@@ -4979,6 +5418,8 @@
       <c r="T179" s="3" t="n"/>
       <c r="U179" s="3" t="n"/>
       <c r="V179" s="3" t="n"/>
+      <c r="W179" s="3" t="n"/>
+      <c r="X179" s="3" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="3" t="n"/>
@@ -5003,6 +5444,8 @@
       <c r="T180" s="3" t="n"/>
       <c r="U180" s="3" t="n"/>
       <c r="V180" s="3" t="n"/>
+      <c r="W180" s="3" t="n"/>
+      <c r="X180" s="3" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="3" t="n"/>
@@ -5027,6 +5470,8 @@
       <c r="T181" s="3" t="n"/>
       <c r="U181" s="3" t="n"/>
       <c r="V181" s="3" t="n"/>
+      <c r="W181" s="3" t="n"/>
+      <c r="X181" s="3" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="3" t="n"/>
@@ -5051,6 +5496,8 @@
       <c r="T182" s="3" t="n"/>
       <c r="U182" s="3" t="n"/>
       <c r="V182" s="3" t="n"/>
+      <c r="W182" s="3" t="n"/>
+      <c r="X182" s="3" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="3" t="n"/>
@@ -5075,6 +5522,8 @@
       <c r="T183" s="3" t="n"/>
       <c r="U183" s="3" t="n"/>
       <c r="V183" s="3" t="n"/>
+      <c r="W183" s="3" t="n"/>
+      <c r="X183" s="3" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="3" t="n"/>
@@ -5099,6 +5548,8 @@
       <c r="T184" s="3" t="n"/>
       <c r="U184" s="3" t="n"/>
       <c r="V184" s="3" t="n"/>
+      <c r="W184" s="3" t="n"/>
+      <c r="X184" s="3" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="3" t="n"/>
@@ -5123,6 +5574,8 @@
       <c r="T185" s="3" t="n"/>
       <c r="U185" s="3" t="n"/>
       <c r="V185" s="3" t="n"/>
+      <c r="W185" s="3" t="n"/>
+      <c r="X185" s="3" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="3" t="n"/>
@@ -5147,6 +5600,8 @@
       <c r="T186" s="3" t="n"/>
       <c r="U186" s="3" t="n"/>
       <c r="V186" s="3" t="n"/>
+      <c r="W186" s="3" t="n"/>
+      <c r="X186" s="3" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="3" t="n"/>
@@ -5171,6 +5626,8 @@
       <c r="T187" s="3" t="n"/>
       <c r="U187" s="3" t="n"/>
       <c r="V187" s="3" t="n"/>
+      <c r="W187" s="3" t="n"/>
+      <c r="X187" s="3" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="3" t="n"/>
@@ -5195,6 +5652,8 @@
       <c r="T188" s="3" t="n"/>
       <c r="U188" s="3" t="n"/>
       <c r="V188" s="3" t="n"/>
+      <c r="W188" s="3" t="n"/>
+      <c r="X188" s="3" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="3" t="n"/>
@@ -5219,6 +5678,8 @@
       <c r="T189" s="3" t="n"/>
       <c r="U189" s="3" t="n"/>
       <c r="V189" s="3" t="n"/>
+      <c r="W189" s="3" t="n"/>
+      <c r="X189" s="3" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="3" t="n"/>
@@ -5243,6 +5704,8 @@
       <c r="T190" s="3" t="n"/>
       <c r="U190" s="3" t="n"/>
       <c r="V190" s="3" t="n"/>
+      <c r="W190" s="3" t="n"/>
+      <c r="X190" s="3" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="3" t="n"/>
@@ -5267,6 +5730,8 @@
       <c r="T191" s="3" t="n"/>
       <c r="U191" s="3" t="n"/>
       <c r="V191" s="3" t="n"/>
+      <c r="W191" s="3" t="n"/>
+      <c r="X191" s="3" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="3" t="n"/>
@@ -5291,6 +5756,8 @@
       <c r="T192" s="3" t="n"/>
       <c r="U192" s="3" t="n"/>
       <c r="V192" s="3" t="n"/>
+      <c r="W192" s="3" t="n"/>
+      <c r="X192" s="3" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="3" t="n"/>
@@ -5315,6 +5782,8 @@
       <c r="T193" s="3" t="n"/>
       <c r="U193" s="3" t="n"/>
       <c r="V193" s="3" t="n"/>
+      <c r="W193" s="3" t="n"/>
+      <c r="X193" s="3" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="3" t="n"/>
@@ -5339,6 +5808,8 @@
       <c r="T194" s="3" t="n"/>
       <c r="U194" s="3" t="n"/>
       <c r="V194" s="3" t="n"/>
+      <c r="W194" s="3" t="n"/>
+      <c r="X194" s="3" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="3" t="n"/>
@@ -5363,6 +5834,8 @@
       <c r="T195" s="3" t="n"/>
       <c r="U195" s="3" t="n"/>
       <c r="V195" s="3" t="n"/>
+      <c r="W195" s="3" t="n"/>
+      <c r="X195" s="3" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="3" t="n"/>
@@ -5387,6 +5860,8 @@
       <c r="T196" s="3" t="n"/>
       <c r="U196" s="3" t="n"/>
       <c r="V196" s="3" t="n"/>
+      <c r="W196" s="3" t="n"/>
+      <c r="X196" s="3" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="3" t="n"/>
@@ -5411,6 +5886,8 @@
       <c r="T197" s="3" t="n"/>
       <c r="U197" s="3" t="n"/>
       <c r="V197" s="3" t="n"/>
+      <c r="W197" s="3" t="n"/>
+      <c r="X197" s="3" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="3" t="n"/>
@@ -5435,6 +5912,8 @@
       <c r="T198" s="3" t="n"/>
       <c r="U198" s="3" t="n"/>
       <c r="V198" s="3" t="n"/>
+      <c r="W198" s="3" t="n"/>
+      <c r="X198" s="3" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="3" t="n"/>
@@ -5459,6 +5938,8 @@
       <c r="T199" s="3" t="n"/>
       <c r="U199" s="3" t="n"/>
       <c r="V199" s="3" t="n"/>
+      <c r="W199" s="3" t="n"/>
+      <c r="X199" s="3" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="3" t="n"/>
@@ -5483,6 +5964,8 @@
       <c r="T200" s="3" t="n"/>
       <c r="U200" s="3" t="n"/>
       <c r="V200" s="3" t="n"/>
+      <c r="W200" s="3" t="n"/>
+      <c r="X200" s="3" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="3" t="n"/>
@@ -5507,6 +5990,8 @@
       <c r="T201" s="3" t="n"/>
       <c r="U201" s="3" t="n"/>
       <c r="V201" s="3" t="n"/>
+      <c r="W201" s="3" t="n"/>
+      <c r="X201" s="3" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="3" t="n"/>
@@ -5531,6 +6016,8 @@
       <c r="T202" s="3" t="n"/>
       <c r="U202" s="3" t="n"/>
       <c r="V202" s="3" t="n"/>
+      <c r="W202" s="3" t="n"/>
+      <c r="X202" s="3" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="3" t="n"/>
@@ -5555,6 +6042,8 @@
       <c r="T203" s="3" t="n"/>
       <c r="U203" s="3" t="n"/>
       <c r="V203" s="3" t="n"/>
+      <c r="W203" s="3" t="n"/>
+      <c r="X203" s="3" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="3" t="n"/>
@@ -5579,6 +6068,8 @@
       <c r="T204" s="3" t="n"/>
       <c r="U204" s="3" t="n"/>
       <c r="V204" s="3" t="n"/>
+      <c r="W204" s="3" t="n"/>
+      <c r="X204" s="3" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="3" t="n"/>
@@ -5603,6 +6094,8 @@
       <c r="T205" s="3" t="n"/>
       <c r="U205" s="3" t="n"/>
       <c r="V205" s="3" t="n"/>
+      <c r="W205" s="3" t="n"/>
+      <c r="X205" s="3" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="3" t="n"/>
@@ -5627,6 +6120,8 @@
       <c r="T206" s="3" t="n"/>
       <c r="U206" s="3" t="n"/>
       <c r="V206" s="3" t="n"/>
+      <c r="W206" s="3" t="n"/>
+      <c r="X206" s="3" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="3" t="n"/>
@@ -5651,6 +6146,8 @@
       <c r="T207" s="3" t="n"/>
       <c r="U207" s="3" t="n"/>
       <c r="V207" s="3" t="n"/>
+      <c r="W207" s="3" t="n"/>
+      <c r="X207" s="3" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="3" t="n"/>
@@ -5675,6 +6172,8 @@
       <c r="T208" s="3" t="n"/>
       <c r="U208" s="3" t="n"/>
       <c r="V208" s="3" t="n"/>
+      <c r="W208" s="3" t="n"/>
+      <c r="X208" s="3" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="3" t="n"/>
@@ -5699,6 +6198,8 @@
       <c r="T209" s="3" t="n"/>
       <c r="U209" s="3" t="n"/>
       <c r="V209" s="3" t="n"/>
+      <c r="W209" s="3" t="n"/>
+      <c r="X209" s="3" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="3" t="n"/>
@@ -5723,6 +6224,8 @@
       <c r="T210" s="3" t="n"/>
       <c r="U210" s="3" t="n"/>
       <c r="V210" s="3" t="n"/>
+      <c r="W210" s="3" t="n"/>
+      <c r="X210" s="3" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="3" t="n"/>
@@ -5747,6 +6250,8 @@
       <c r="T211" s="3" t="n"/>
       <c r="U211" s="3" t="n"/>
       <c r="V211" s="3" t="n"/>
+      <c r="W211" s="3" t="n"/>
+      <c r="X211" s="3" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="3" t="n"/>
@@ -5771,6 +6276,8 @@
       <c r="T212" s="3" t="n"/>
       <c r="U212" s="3" t="n"/>
       <c r="V212" s="3" t="n"/>
+      <c r="W212" s="3" t="n"/>
+      <c r="X212" s="3" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="3" t="n"/>
@@ -5795,6 +6302,8 @@
       <c r="T213" s="3" t="n"/>
       <c r="U213" s="3" t="n"/>
       <c r="V213" s="3" t="n"/>
+      <c r="W213" s="3" t="n"/>
+      <c r="X213" s="3" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="3" t="n"/>
@@ -5819,6 +6328,8 @@
       <c r="T214" s="3" t="n"/>
       <c r="U214" s="3" t="n"/>
       <c r="V214" s="3" t="n"/>
+      <c r="W214" s="3" t="n"/>
+      <c r="X214" s="3" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="3" t="n"/>
@@ -5843,6 +6354,8 @@
       <c r="T215" s="3" t="n"/>
       <c r="U215" s="3" t="n"/>
       <c r="V215" s="3" t="n"/>
+      <c r="W215" s="3" t="n"/>
+      <c r="X215" s="3" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="3" t="n"/>
@@ -5867,6 +6380,8 @@
       <c r="T216" s="3" t="n"/>
       <c r="U216" s="3" t="n"/>
       <c r="V216" s="3" t="n"/>
+      <c r="W216" s="3" t="n"/>
+      <c r="X216" s="3" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="3" t="n"/>
@@ -5891,6 +6406,8 @@
       <c r="T217" s="3" t="n"/>
       <c r="U217" s="3" t="n"/>
       <c r="V217" s="3" t="n"/>
+      <c r="W217" s="3" t="n"/>
+      <c r="X217" s="3" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="3" t="n"/>
@@ -5915,6 +6432,8 @@
       <c r="T218" s="3" t="n"/>
       <c r="U218" s="3" t="n"/>
       <c r="V218" s="3" t="n"/>
+      <c r="W218" s="3" t="n"/>
+      <c r="X218" s="3" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="3" t="n"/>
@@ -5939,6 +6458,8 @@
       <c r="T219" s="3" t="n"/>
       <c r="U219" s="3" t="n"/>
       <c r="V219" s="3" t="n"/>
+      <c r="W219" s="3" t="n"/>
+      <c r="X219" s="3" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="3" t="n"/>
@@ -5963,6 +6484,8 @@
       <c r="T220" s="3" t="n"/>
       <c r="U220" s="3" t="n"/>
       <c r="V220" s="3" t="n"/>
+      <c r="W220" s="3" t="n"/>
+      <c r="X220" s="3" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="3" t="n"/>
@@ -5987,6 +6510,8 @@
       <c r="T221" s="3" t="n"/>
       <c r="U221" s="3" t="n"/>
       <c r="V221" s="3" t="n"/>
+      <c r="W221" s="3" t="n"/>
+      <c r="X221" s="3" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="3" t="n"/>
@@ -6011,6 +6536,8 @@
       <c r="T222" s="3" t="n"/>
       <c r="U222" s="3" t="n"/>
       <c r="V222" s="3" t="n"/>
+      <c r="W222" s="3" t="n"/>
+      <c r="X222" s="3" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="3" t="n"/>
@@ -6035,6 +6562,8 @@
       <c r="T223" s="3" t="n"/>
       <c r="U223" s="3" t="n"/>
       <c r="V223" s="3" t="n"/>
+      <c r="W223" s="3" t="n"/>
+      <c r="X223" s="3" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="3" t="n"/>
@@ -6059,6 +6588,8 @@
       <c r="T224" s="3" t="n"/>
       <c r="U224" s="3" t="n"/>
       <c r="V224" s="3" t="n"/>
+      <c r="W224" s="3" t="n"/>
+      <c r="X224" s="3" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="3" t="n"/>
@@ -6083,6 +6614,8 @@
       <c r="T225" s="3" t="n"/>
       <c r="U225" s="3" t="n"/>
       <c r="V225" s="3" t="n"/>
+      <c r="W225" s="3" t="n"/>
+      <c r="X225" s="3" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="3" t="n"/>
@@ -6107,6 +6640,8 @@
       <c r="T226" s="3" t="n"/>
       <c r="U226" s="3" t="n"/>
       <c r="V226" s="3" t="n"/>
+      <c r="W226" s="3" t="n"/>
+      <c r="X226" s="3" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="3" t="n"/>
@@ -6131,6 +6666,8 @@
       <c r="T227" s="3" t="n"/>
       <c r="U227" s="3" t="n"/>
       <c r="V227" s="3" t="n"/>
+      <c r="W227" s="3" t="n"/>
+      <c r="X227" s="3" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="3" t="n"/>
@@ -6155,6 +6692,8 @@
       <c r="T228" s="3" t="n"/>
       <c r="U228" s="3" t="n"/>
       <c r="V228" s="3" t="n"/>
+      <c r="W228" s="3" t="n"/>
+      <c r="X228" s="3" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="3" t="n"/>
@@ -6179,6 +6718,8 @@
       <c r="T229" s="3" t="n"/>
       <c r="U229" s="3" t="n"/>
       <c r="V229" s="3" t="n"/>
+      <c r="W229" s="3" t="n"/>
+      <c r="X229" s="3" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="3" t="n"/>
@@ -6203,6 +6744,8 @@
       <c r="T230" s="3" t="n"/>
       <c r="U230" s="3" t="n"/>
       <c r="V230" s="3" t="n"/>
+      <c r="W230" s="3" t="n"/>
+      <c r="X230" s="3" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="3" t="n"/>
@@ -6227,6 +6770,8 @@
       <c r="T231" s="3" t="n"/>
       <c r="U231" s="3" t="n"/>
       <c r="V231" s="3" t="n"/>
+      <c r="W231" s="3" t="n"/>
+      <c r="X231" s="3" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="3" t="n"/>
@@ -6251,6 +6796,8 @@
       <c r="T232" s="3" t="n"/>
       <c r="U232" s="3" t="n"/>
       <c r="V232" s="3" t="n"/>
+      <c r="W232" s="3" t="n"/>
+      <c r="X232" s="3" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="3" t="n"/>
@@ -6275,6 +6822,8 @@
       <c r="T233" s="3" t="n"/>
       <c r="U233" s="3" t="n"/>
       <c r="V233" s="3" t="n"/>
+      <c r="W233" s="3" t="n"/>
+      <c r="X233" s="3" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="3" t="n"/>
@@ -6299,6 +6848,8 @@
       <c r="T234" s="3" t="n"/>
       <c r="U234" s="3" t="n"/>
       <c r="V234" s="3" t="n"/>
+      <c r="W234" s="3" t="n"/>
+      <c r="X234" s="3" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="3" t="n"/>
@@ -6323,6 +6874,8 @@
       <c r="T235" s="3" t="n"/>
       <c r="U235" s="3" t="n"/>
       <c r="V235" s="3" t="n"/>
+      <c r="W235" s="3" t="n"/>
+      <c r="X235" s="3" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="3" t="n"/>
@@ -6347,6 +6900,8 @@
       <c r="T236" s="3" t="n"/>
       <c r="U236" s="3" t="n"/>
       <c r="V236" s="3" t="n"/>
+      <c r="W236" s="3" t="n"/>
+      <c r="X236" s="3" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="3" t="n"/>
@@ -6371,6 +6926,8 @@
       <c r="T237" s="3" t="n"/>
       <c r="U237" s="3" t="n"/>
       <c r="V237" s="3" t="n"/>
+      <c r="W237" s="3" t="n"/>
+      <c r="X237" s="3" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="3" t="n"/>
@@ -6395,6 +6952,8 @@
       <c r="T238" s="3" t="n"/>
       <c r="U238" s="3" t="n"/>
       <c r="V238" s="3" t="n"/>
+      <c r="W238" s="3" t="n"/>
+      <c r="X238" s="3" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="3" t="n"/>
@@ -6419,6 +6978,8 @@
       <c r="T239" s="3" t="n"/>
       <c r="U239" s="3" t="n"/>
       <c r="V239" s="3" t="n"/>
+      <c r="W239" s="3" t="n"/>
+      <c r="X239" s="3" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="3" t="n"/>
@@ -6443,6 +7004,8 @@
       <c r="T240" s="3" t="n"/>
       <c r="U240" s="3" t="n"/>
       <c r="V240" s="3" t="n"/>
+      <c r="W240" s="3" t="n"/>
+      <c r="X240" s="3" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="3" t="n"/>
@@ -6467,6 +7030,8 @@
       <c r="T241" s="3" t="n"/>
       <c r="U241" s="3" t="n"/>
       <c r="V241" s="3" t="n"/>
+      <c r="W241" s="3" t="n"/>
+      <c r="X241" s="3" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="3" t="n"/>
@@ -6491,6 +7056,8 @@
       <c r="T242" s="3" t="n"/>
       <c r="U242" s="3" t="n"/>
       <c r="V242" s="3" t="n"/>
+      <c r="W242" s="3" t="n"/>
+      <c r="X242" s="3" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="3" t="n"/>
@@ -6515,6 +7082,8 @@
       <c r="T243" s="3" t="n"/>
       <c r="U243" s="3" t="n"/>
       <c r="V243" s="3" t="n"/>
+      <c r="W243" s="3" t="n"/>
+      <c r="X243" s="3" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="3" t="n"/>
@@ -6539,6 +7108,8 @@
       <c r="T244" s="3" t="n"/>
       <c r="U244" s="3" t="n"/>
       <c r="V244" s="3" t="n"/>
+      <c r="W244" s="3" t="n"/>
+      <c r="X244" s="3" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="3" t="n"/>
@@ -6563,6 +7134,8 @@
       <c r="T245" s="3" t="n"/>
       <c r="U245" s="3" t="n"/>
       <c r="V245" s="3" t="n"/>
+      <c r="W245" s="3" t="n"/>
+      <c r="X245" s="3" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="3" t="n"/>
@@ -6587,6 +7160,8 @@
       <c r="T246" s="3" t="n"/>
       <c r="U246" s="3" t="n"/>
       <c r="V246" s="3" t="n"/>
+      <c r="W246" s="3" t="n"/>
+      <c r="X246" s="3" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="3" t="n"/>
@@ -6611,6 +7186,8 @@
       <c r="T247" s="3" t="n"/>
       <c r="U247" s="3" t="n"/>
       <c r="V247" s="3" t="n"/>
+      <c r="W247" s="3" t="n"/>
+      <c r="X247" s="3" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="3" t="n"/>
@@ -6635,6 +7212,8 @@
       <c r="T248" s="3" t="n"/>
       <c r="U248" s="3" t="n"/>
       <c r="V248" s="3" t="n"/>
+      <c r="W248" s="3" t="n"/>
+      <c r="X248" s="3" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="3" t="n"/>
@@ -6659,6 +7238,8 @@
       <c r="T249" s="3" t="n"/>
       <c r="U249" s="3" t="n"/>
       <c r="V249" s="3" t="n"/>
+      <c r="W249" s="3" t="n"/>
+      <c r="X249" s="3" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="3" t="n"/>
@@ -6683,6 +7264,8 @@
       <c r="T250" s="3" t="n"/>
       <c r="U250" s="3" t="n"/>
       <c r="V250" s="3" t="n"/>
+      <c r="W250" s="3" t="n"/>
+      <c r="X250" s="3" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="3" t="n"/>
@@ -6707,6 +7290,8 @@
       <c r="T251" s="3" t="n"/>
       <c r="U251" s="3" t="n"/>
       <c r="V251" s="3" t="n"/>
+      <c r="W251" s="3" t="n"/>
+      <c r="X251" s="3" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="3" t="n"/>
@@ -6731,6 +7316,8 @@
       <c r="T252" s="3" t="n"/>
       <c r="U252" s="3" t="n"/>
       <c r="V252" s="3" t="n"/>
+      <c r="W252" s="3" t="n"/>
+      <c r="X252" s="3" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="3" t="n"/>
@@ -6755,6 +7342,8 @@
       <c r="T253" s="3" t="n"/>
       <c r="U253" s="3" t="n"/>
       <c r="V253" s="3" t="n"/>
+      <c r="W253" s="3" t="n"/>
+      <c r="X253" s="3" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="3" t="n"/>
@@ -6779,6 +7368,8 @@
       <c r="T254" s="3" t="n"/>
       <c r="U254" s="3" t="n"/>
       <c r="V254" s="3" t="n"/>
+      <c r="W254" s="3" t="n"/>
+      <c r="X254" s="3" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="3" t="n"/>
@@ -6803,6 +7394,8 @@
       <c r="T255" s="3" t="n"/>
       <c r="U255" s="3" t="n"/>
       <c r="V255" s="3" t="n"/>
+      <c r="W255" s="3" t="n"/>
+      <c r="X255" s="3" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="3" t="n"/>
@@ -6827,6 +7420,8 @@
       <c r="T256" s="3" t="n"/>
       <c r="U256" s="3" t="n"/>
       <c r="V256" s="3" t="n"/>
+      <c r="W256" s="3" t="n"/>
+      <c r="X256" s="3" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="3" t="n"/>
@@ -6851,6 +7446,8 @@
       <c r="T257" s="3" t="n"/>
       <c r="U257" s="3" t="n"/>
       <c r="V257" s="3" t="n"/>
+      <c r="W257" s="3" t="n"/>
+      <c r="X257" s="3" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="3" t="n"/>
@@ -6875,6 +7472,8 @@
       <c r="T258" s="3" t="n"/>
       <c r="U258" s="3" t="n"/>
       <c r="V258" s="3" t="n"/>
+      <c r="W258" s="3" t="n"/>
+      <c r="X258" s="3" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="3" t="n"/>
@@ -6899,6 +7498,8 @@
       <c r="T259" s="3" t="n"/>
       <c r="U259" s="3" t="n"/>
       <c r="V259" s="3" t="n"/>
+      <c r="W259" s="3" t="n"/>
+      <c r="X259" s="3" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="3" t="n"/>
@@ -6923,6 +7524,8 @@
       <c r="T260" s="3" t="n"/>
       <c r="U260" s="3" t="n"/>
       <c r="V260" s="3" t="n"/>
+      <c r="W260" s="3" t="n"/>
+      <c r="X260" s="3" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="3" t="n"/>
@@ -6947,6 +7550,8 @@
       <c r="T261" s="3" t="n"/>
       <c r="U261" s="3" t="n"/>
       <c r="V261" s="3" t="n"/>
+      <c r="W261" s="3" t="n"/>
+      <c r="X261" s="3" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="3" t="n"/>
@@ -6971,6 +7576,8 @@
       <c r="T262" s="3" t="n"/>
       <c r="U262" s="3" t="n"/>
       <c r="V262" s="3" t="n"/>
+      <c r="W262" s="3" t="n"/>
+      <c r="X262" s="3" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="3" t="n"/>
@@ -6995,6 +7602,8 @@
       <c r="T263" s="3" t="n"/>
       <c r="U263" s="3" t="n"/>
       <c r="V263" s="3" t="n"/>
+      <c r="W263" s="3" t="n"/>
+      <c r="X263" s="3" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="3" t="n"/>
@@ -7019,6 +7628,8 @@
       <c r="T264" s="3" t="n"/>
       <c r="U264" s="3" t="n"/>
       <c r="V264" s="3" t="n"/>
+      <c r="W264" s="3" t="n"/>
+      <c r="X264" s="3" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="3" t="n"/>
@@ -7043,6 +7654,8 @@
       <c r="T265" s="3" t="n"/>
       <c r="U265" s="3" t="n"/>
       <c r="V265" s="3" t="n"/>
+      <c r="W265" s="3" t="n"/>
+      <c r="X265" s="3" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="3" t="n"/>
@@ -7067,6 +7680,8 @@
       <c r="T266" s="3" t="n"/>
       <c r="U266" s="3" t="n"/>
       <c r="V266" s="3" t="n"/>
+      <c r="W266" s="3" t="n"/>
+      <c r="X266" s="3" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="3" t="n"/>
@@ -7091,6 +7706,8 @@
       <c r="T267" s="3" t="n"/>
       <c r="U267" s="3" t="n"/>
       <c r="V267" s="3" t="n"/>
+      <c r="W267" s="3" t="n"/>
+      <c r="X267" s="3" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="3" t="n"/>
@@ -7115,6 +7732,8 @@
       <c r="T268" s="3" t="n"/>
       <c r="U268" s="3" t="n"/>
       <c r="V268" s="3" t="n"/>
+      <c r="W268" s="3" t="n"/>
+      <c r="X268" s="3" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="3" t="n"/>
@@ -7139,6 +7758,8 @@
       <c r="T269" s="3" t="n"/>
       <c r="U269" s="3" t="n"/>
       <c r="V269" s="3" t="n"/>
+      <c r="W269" s="3" t="n"/>
+      <c r="X269" s="3" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="3" t="n"/>
@@ -7163,6 +7784,8 @@
       <c r="T270" s="3" t="n"/>
       <c r="U270" s="3" t="n"/>
       <c r="V270" s="3" t="n"/>
+      <c r="W270" s="3" t="n"/>
+      <c r="X270" s="3" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="3" t="n"/>
@@ -7187,6 +7810,8 @@
       <c r="T271" s="3" t="n"/>
       <c r="U271" s="3" t="n"/>
       <c r="V271" s="3" t="n"/>
+      <c r="W271" s="3" t="n"/>
+      <c r="X271" s="3" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="3" t="n"/>
@@ -7211,6 +7836,8 @@
       <c r="T272" s="3" t="n"/>
       <c r="U272" s="3" t="n"/>
       <c r="V272" s="3" t="n"/>
+      <c r="W272" s="3" t="n"/>
+      <c r="X272" s="3" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="3" t="n"/>
@@ -7235,6 +7862,8 @@
       <c r="T273" s="3" t="n"/>
       <c r="U273" s="3" t="n"/>
       <c r="V273" s="3" t="n"/>
+      <c r="W273" s="3" t="n"/>
+      <c r="X273" s="3" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="3" t="n"/>
@@ -7259,6 +7888,8 @@
       <c r="T274" s="3" t="n"/>
       <c r="U274" s="3" t="n"/>
       <c r="V274" s="3" t="n"/>
+      <c r="W274" s="3" t="n"/>
+      <c r="X274" s="3" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="3" t="n"/>
@@ -7283,6 +7914,8 @@
       <c r="T275" s="3" t="n"/>
       <c r="U275" s="3" t="n"/>
       <c r="V275" s="3" t="n"/>
+      <c r="W275" s="3" t="n"/>
+      <c r="X275" s="3" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="3" t="n"/>
@@ -7307,6 +7940,8 @@
       <c r="T276" s="3" t="n"/>
       <c r="U276" s="3" t="n"/>
       <c r="V276" s="3" t="n"/>
+      <c r="W276" s="3" t="n"/>
+      <c r="X276" s="3" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="3" t="n"/>
@@ -7331,6 +7966,8 @@
       <c r="T277" s="3" t="n"/>
       <c r="U277" s="3" t="n"/>
       <c r="V277" s="3" t="n"/>
+      <c r="W277" s="3" t="n"/>
+      <c r="X277" s="3" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="3" t="n"/>
@@ -7355,6 +7992,8 @@
       <c r="T278" s="3" t="n"/>
       <c r="U278" s="3" t="n"/>
       <c r="V278" s="3" t="n"/>
+      <c r="W278" s="3" t="n"/>
+      <c r="X278" s="3" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="3" t="n"/>
@@ -7379,6 +8018,8 @@
       <c r="T279" s="3" t="n"/>
       <c r="U279" s="3" t="n"/>
       <c r="V279" s="3" t="n"/>
+      <c r="W279" s="3" t="n"/>
+      <c r="X279" s="3" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="3" t="n"/>
@@ -7403,6 +8044,8 @@
       <c r="T280" s="3" t="n"/>
       <c r="U280" s="3" t="n"/>
       <c r="V280" s="3" t="n"/>
+      <c r="W280" s="3" t="n"/>
+      <c r="X280" s="3" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="3" t="n"/>
@@ -7427,6 +8070,8 @@
       <c r="T281" s="3" t="n"/>
       <c r="U281" s="3" t="n"/>
       <c r="V281" s="3" t="n"/>
+      <c r="W281" s="3" t="n"/>
+      <c r="X281" s="3" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="3" t="n"/>
@@ -7451,6 +8096,8 @@
       <c r="T282" s="3" t="n"/>
       <c r="U282" s="3" t="n"/>
       <c r="V282" s="3" t="n"/>
+      <c r="W282" s="3" t="n"/>
+      <c r="X282" s="3" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="3" t="n"/>
@@ -7475,6 +8122,8 @@
       <c r="T283" s="3" t="n"/>
       <c r="U283" s="3" t="n"/>
       <c r="V283" s="3" t="n"/>
+      <c r="W283" s="3" t="n"/>
+      <c r="X283" s="3" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="3" t="n"/>
@@ -7499,6 +8148,8 @@
       <c r="T284" s="3" t="n"/>
       <c r="U284" s="3" t="n"/>
       <c r="V284" s="3" t="n"/>
+      <c r="W284" s="3" t="n"/>
+      <c r="X284" s="3" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="3" t="n"/>
@@ -7523,6 +8174,8 @@
       <c r="T285" s="3" t="n"/>
       <c r="U285" s="3" t="n"/>
       <c r="V285" s="3" t="n"/>
+      <c r="W285" s="3" t="n"/>
+      <c r="X285" s="3" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="3" t="n"/>
@@ -7547,6 +8200,8 @@
       <c r="T286" s="3" t="n"/>
       <c r="U286" s="3" t="n"/>
       <c r="V286" s="3" t="n"/>
+      <c r="W286" s="3" t="n"/>
+      <c r="X286" s="3" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="3" t="n"/>
@@ -7571,6 +8226,8 @@
       <c r="T287" s="3" t="n"/>
       <c r="U287" s="3" t="n"/>
       <c r="V287" s="3" t="n"/>
+      <c r="W287" s="3" t="n"/>
+      <c r="X287" s="3" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="3" t="n"/>
@@ -7595,6 +8252,8 @@
       <c r="T288" s="3" t="n"/>
       <c r="U288" s="3" t="n"/>
       <c r="V288" s="3" t="n"/>
+      <c r="W288" s="3" t="n"/>
+      <c r="X288" s="3" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="3" t="n"/>
@@ -7619,6 +8278,8 @@
       <c r="T289" s="3" t="n"/>
       <c r="U289" s="3" t="n"/>
       <c r="V289" s="3" t="n"/>
+      <c r="W289" s="3" t="n"/>
+      <c r="X289" s="3" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="3" t="n"/>
@@ -7643,6 +8304,8 @@
       <c r="T290" s="3" t="n"/>
       <c r="U290" s="3" t="n"/>
       <c r="V290" s="3" t="n"/>
+      <c r="W290" s="3" t="n"/>
+      <c r="X290" s="3" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="3" t="n"/>
@@ -7667,6 +8330,8 @@
       <c r="T291" s="3" t="n"/>
       <c r="U291" s="3" t="n"/>
       <c r="V291" s="3" t="n"/>
+      <c r="W291" s="3" t="n"/>
+      <c r="X291" s="3" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="3" t="n"/>
@@ -7691,6 +8356,8 @@
       <c r="T292" s="3" t="n"/>
       <c r="U292" s="3" t="n"/>
       <c r="V292" s="3" t="n"/>
+      <c r="W292" s="3" t="n"/>
+      <c r="X292" s="3" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="3" t="n"/>
@@ -7715,6 +8382,8 @@
       <c r="T293" s="3" t="n"/>
       <c r="U293" s="3" t="n"/>
       <c r="V293" s="3" t="n"/>
+      <c r="W293" s="3" t="n"/>
+      <c r="X293" s="3" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="3" t="n"/>
@@ -7739,6 +8408,8 @@
       <c r="T294" s="3" t="n"/>
       <c r="U294" s="3" t="n"/>
       <c r="V294" s="3" t="n"/>
+      <c r="W294" s="3" t="n"/>
+      <c r="X294" s="3" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="3" t="n"/>
@@ -7763,6 +8434,8 @@
       <c r="T295" s="3" t="n"/>
       <c r="U295" s="3" t="n"/>
       <c r="V295" s="3" t="n"/>
+      <c r="W295" s="3" t="n"/>
+      <c r="X295" s="3" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="3" t="n"/>
@@ -7787,6 +8460,8 @@
       <c r="T296" s="3" t="n"/>
       <c r="U296" s="3" t="n"/>
       <c r="V296" s="3" t="n"/>
+      <c r="W296" s="3" t="n"/>
+      <c r="X296" s="3" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="3" t="n"/>
@@ -7811,6 +8486,8 @@
       <c r="T297" s="3" t="n"/>
       <c r="U297" s="3" t="n"/>
       <c r="V297" s="3" t="n"/>
+      <c r="W297" s="3" t="n"/>
+      <c r="X297" s="3" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="3" t="n"/>
@@ -7835,6 +8512,8 @@
       <c r="T298" s="3" t="n"/>
       <c r="U298" s="3" t="n"/>
       <c r="V298" s="3" t="n"/>
+      <c r="W298" s="3" t="n"/>
+      <c r="X298" s="3" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="3" t="n"/>
@@ -7859,6 +8538,8 @@
       <c r="T299" s="3" t="n"/>
       <c r="U299" s="3" t="n"/>
       <c r="V299" s="3" t="n"/>
+      <c r="W299" s="3" t="n"/>
+      <c r="X299" s="3" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="3" t="n"/>
@@ -7883,6 +8564,8 @@
       <c r="T300" s="3" t="n"/>
       <c r="U300" s="3" t="n"/>
       <c r="V300" s="3" t="n"/>
+      <c r="W300" s="3" t="n"/>
+      <c r="X300" s="3" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="3" t="n"/>
@@ -7907,6 +8590,8 @@
       <c r="T301" s="3" t="n"/>
       <c r="U301" s="3" t="n"/>
       <c r="V301" s="3" t="n"/>
+      <c r="W301" s="3" t="n"/>
+      <c r="X301" s="3" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="3" t="n"/>
@@ -7931,6 +8616,8 @@
       <c r="T302" s="3" t="n"/>
       <c r="U302" s="3" t="n"/>
       <c r="V302" s="3" t="n"/>
+      <c r="W302" s="3" t="n"/>
+      <c r="X302" s="3" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="3" t="n"/>
@@ -7955,6 +8642,8 @@
       <c r="T303" s="3" t="n"/>
       <c r="U303" s="3" t="n"/>
       <c r="V303" s="3" t="n"/>
+      <c r="W303" s="3" t="n"/>
+      <c r="X303" s="3" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="3" t="n"/>
@@ -7979,6 +8668,8 @@
       <c r="T304" s="3" t="n"/>
       <c r="U304" s="3" t="n"/>
       <c r="V304" s="3" t="n"/>
+      <c r="W304" s="3" t="n"/>
+      <c r="X304" s="3" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="3" t="n"/>
@@ -8003,6 +8694,8 @@
       <c r="T305" s="3" t="n"/>
       <c r="U305" s="3" t="n"/>
       <c r="V305" s="3" t="n"/>
+      <c r="W305" s="3" t="n"/>
+      <c r="X305" s="3" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="3" t="n"/>
@@ -8027,6 +8720,8 @@
       <c r="T306" s="3" t="n"/>
       <c r="U306" s="3" t="n"/>
       <c r="V306" s="3" t="n"/>
+      <c r="W306" s="3" t="n"/>
+      <c r="X306" s="3" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="3" t="n"/>
@@ -8051,6 +8746,8 @@
       <c r="T307" s="3" t="n"/>
       <c r="U307" s="3" t="n"/>
       <c r="V307" s="3" t="n"/>
+      <c r="W307" s="3" t="n"/>
+      <c r="X307" s="3" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="3" t="n"/>
@@ -8075,6 +8772,8 @@
       <c r="T308" s="3" t="n"/>
       <c r="U308" s="3" t="n"/>
       <c r="V308" s="3" t="n"/>
+      <c r="W308" s="3" t="n"/>
+      <c r="X308" s="3" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="3" t="n"/>
@@ -8099,6 +8798,8 @@
       <c r="T309" s="3" t="n"/>
       <c r="U309" s="3" t="n"/>
       <c r="V309" s="3" t="n"/>
+      <c r="W309" s="3" t="n"/>
+      <c r="X309" s="3" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="3" t="n"/>
@@ -8123,6 +8824,8 @@
       <c r="T310" s="3" t="n"/>
       <c r="U310" s="3" t="n"/>
       <c r="V310" s="3" t="n"/>
+      <c r="W310" s="3" t="n"/>
+      <c r="X310" s="3" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="3" t="n"/>
@@ -8147,6 +8850,8 @@
       <c r="T311" s="3" t="n"/>
       <c r="U311" s="3" t="n"/>
       <c r="V311" s="3" t="n"/>
+      <c r="W311" s="3" t="n"/>
+      <c r="X311" s="3" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="3" t="n"/>
@@ -8171,6 +8876,8 @@
       <c r="T312" s="3" t="n"/>
       <c r="U312" s="3" t="n"/>
       <c r="V312" s="3" t="n"/>
+      <c r="W312" s="3" t="n"/>
+      <c r="X312" s="3" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="3" t="n"/>
@@ -8195,6 +8902,8 @@
       <c r="T313" s="3" t="n"/>
       <c r="U313" s="3" t="n"/>
       <c r="V313" s="3" t="n"/>
+      <c r="W313" s="3" t="n"/>
+      <c r="X313" s="3" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="3" t="n"/>
@@ -8219,6 +8928,8 @@
       <c r="T314" s="3" t="n"/>
       <c r="U314" s="3" t="n"/>
       <c r="V314" s="3" t="n"/>
+      <c r="W314" s="3" t="n"/>
+      <c r="X314" s="3" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="3" t="n"/>
@@ -8243,6 +8954,8 @@
       <c r="T315" s="3" t="n"/>
       <c r="U315" s="3" t="n"/>
       <c r="V315" s="3" t="n"/>
+      <c r="W315" s="3" t="n"/>
+      <c r="X315" s="3" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="3" t="n"/>
@@ -8267,6 +8980,8 @@
       <c r="T316" s="3" t="n"/>
       <c r="U316" s="3" t="n"/>
       <c r="V316" s="3" t="n"/>
+      <c r="W316" s="3" t="n"/>
+      <c r="X316" s="3" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="3" t="n"/>
@@ -8291,6 +9006,8 @@
       <c r="T317" s="3" t="n"/>
       <c r="U317" s="3" t="n"/>
       <c r="V317" s="3" t="n"/>
+      <c r="W317" s="3" t="n"/>
+      <c r="X317" s="3" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="3" t="n"/>
@@ -8315,6 +9032,8 @@
       <c r="T318" s="3" t="n"/>
       <c r="U318" s="3" t="n"/>
       <c r="V318" s="3" t="n"/>
+      <c r="W318" s="3" t="n"/>
+      <c r="X318" s="3" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="3" t="n"/>
@@ -8339,6 +9058,8 @@
       <c r="T319" s="3" t="n"/>
       <c r="U319" s="3" t="n"/>
       <c r="V319" s="3" t="n"/>
+      <c r="W319" s="3" t="n"/>
+      <c r="X319" s="3" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="3" t="n"/>
@@ -8363,6 +9084,8 @@
       <c r="T320" s="3" t="n"/>
       <c r="U320" s="3" t="n"/>
       <c r="V320" s="3" t="n"/>
+      <c r="W320" s="3" t="n"/>
+      <c r="X320" s="3" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="3" t="n"/>
@@ -8387,6 +9110,8 @@
       <c r="T321" s="3" t="n"/>
       <c r="U321" s="3" t="n"/>
       <c r="V321" s="3" t="n"/>
+      <c r="W321" s="3" t="n"/>
+      <c r="X321" s="3" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="3" t="n"/>
@@ -8411,6 +9136,8 @@
       <c r="T322" s="3" t="n"/>
       <c r="U322" s="3" t="n"/>
       <c r="V322" s="3" t="n"/>
+      <c r="W322" s="3" t="n"/>
+      <c r="X322" s="3" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="3" t="n"/>
@@ -8435,6 +9162,8 @@
       <c r="T323" s="3" t="n"/>
       <c r="U323" s="3" t="n"/>
       <c r="V323" s="3" t="n"/>
+      <c r="W323" s="3" t="n"/>
+      <c r="X323" s="3" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="3" t="n"/>
@@ -8459,6 +9188,8 @@
       <c r="T324" s="3" t="n"/>
       <c r="U324" s="3" t="n"/>
       <c r="V324" s="3" t="n"/>
+      <c r="W324" s="3" t="n"/>
+      <c r="X324" s="3" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="3" t="n"/>
@@ -8483,6 +9214,8 @@
       <c r="T325" s="3" t="n"/>
       <c r="U325" s="3" t="n"/>
       <c r="V325" s="3" t="n"/>
+      <c r="W325" s="3" t="n"/>
+      <c r="X325" s="3" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="3" t="n"/>
@@ -8507,6 +9240,8 @@
       <c r="T326" s="3" t="n"/>
       <c r="U326" s="3" t="n"/>
       <c r="V326" s="3" t="n"/>
+      <c r="W326" s="3" t="n"/>
+      <c r="X326" s="3" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="3" t="n"/>
@@ -8531,6 +9266,8 @@
       <c r="T327" s="3" t="n"/>
       <c r="U327" s="3" t="n"/>
       <c r="V327" s="3" t="n"/>
+      <c r="W327" s="3" t="n"/>
+      <c r="X327" s="3" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="3" t="n"/>
@@ -8555,6 +9292,8 @@
       <c r="T328" s="3" t="n"/>
       <c r="U328" s="3" t="n"/>
       <c r="V328" s="3" t="n"/>
+      <c r="W328" s="3" t="n"/>
+      <c r="X328" s="3" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="3" t="n"/>
@@ -8579,6 +9318,8 @@
       <c r="T329" s="3" t="n"/>
       <c r="U329" s="3" t="n"/>
       <c r="V329" s="3" t="n"/>
+      <c r="W329" s="3" t="n"/>
+      <c r="X329" s="3" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="3" t="n"/>
@@ -8603,6 +9344,8 @@
       <c r="T330" s="3" t="n"/>
       <c r="U330" s="3" t="n"/>
       <c r="V330" s="3" t="n"/>
+      <c r="W330" s="3" t="n"/>
+      <c r="X330" s="3" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="3" t="n"/>
@@ -8627,6 +9370,8 @@
       <c r="T331" s="3" t="n"/>
       <c r="U331" s="3" t="n"/>
       <c r="V331" s="3" t="n"/>
+      <c r="W331" s="3" t="n"/>
+      <c r="X331" s="3" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="3" t="n"/>
@@ -8651,6 +9396,8 @@
       <c r="T332" s="3" t="n"/>
       <c r="U332" s="3" t="n"/>
       <c r="V332" s="3" t="n"/>
+      <c r="W332" s="3" t="n"/>
+      <c r="X332" s="3" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="3" t="n"/>
@@ -8675,6 +9422,8 @@
       <c r="T333" s="3" t="n"/>
       <c r="U333" s="3" t="n"/>
       <c r="V333" s="3" t="n"/>
+      <c r="W333" s="3" t="n"/>
+      <c r="X333" s="3" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="3" t="n"/>
@@ -8699,6 +9448,8 @@
       <c r="T334" s="3" t="n"/>
       <c r="U334" s="3" t="n"/>
       <c r="V334" s="3" t="n"/>
+      <c r="W334" s="3" t="n"/>
+      <c r="X334" s="3" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="3" t="n"/>
@@ -8723,6 +9474,8 @@
       <c r="T335" s="3" t="n"/>
       <c r="U335" s="3" t="n"/>
       <c r="V335" s="3" t="n"/>
+      <c r="W335" s="3" t="n"/>
+      <c r="X335" s="3" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="3" t="n"/>
@@ -8747,6 +9500,8 @@
       <c r="T336" s="3" t="n"/>
       <c r="U336" s="3" t="n"/>
       <c r="V336" s="3" t="n"/>
+      <c r="W336" s="3" t="n"/>
+      <c r="X336" s="3" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="3" t="n"/>
@@ -8771,6 +9526,8 @@
       <c r="T337" s="3" t="n"/>
       <c r="U337" s="3" t="n"/>
       <c r="V337" s="3" t="n"/>
+      <c r="W337" s="3" t="n"/>
+      <c r="X337" s="3" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="3" t="n"/>
@@ -8795,6 +9552,8 @@
       <c r="T338" s="3" t="n"/>
       <c r="U338" s="3" t="n"/>
       <c r="V338" s="3" t="n"/>
+      <c r="W338" s="3" t="n"/>
+      <c r="X338" s="3" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="3" t="n"/>
@@ -8819,6 +9578,8 @@
       <c r="T339" s="3" t="n"/>
       <c r="U339" s="3" t="n"/>
       <c r="V339" s="3" t="n"/>
+      <c r="W339" s="3" t="n"/>
+      <c r="X339" s="3" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="3" t="n"/>
@@ -8843,6 +9604,8 @@
       <c r="T340" s="3" t="n"/>
       <c r="U340" s="3" t="n"/>
       <c r="V340" s="3" t="n"/>
+      <c r="W340" s="3" t="n"/>
+      <c r="X340" s="3" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="3" t="n"/>
@@ -8867,6 +9630,8 @@
       <c r="T341" s="3" t="n"/>
       <c r="U341" s="3" t="n"/>
       <c r="V341" s="3" t="n"/>
+      <c r="W341" s="3" t="n"/>
+      <c r="X341" s="3" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="3" t="n"/>
@@ -8891,6 +9656,8 @@
       <c r="T342" s="3" t="n"/>
       <c r="U342" s="3" t="n"/>
       <c r="V342" s="3" t="n"/>
+      <c r="W342" s="3" t="n"/>
+      <c r="X342" s="3" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="3" t="n"/>
@@ -8915,6 +9682,8 @@
       <c r="T343" s="3" t="n"/>
       <c r="U343" s="3" t="n"/>
       <c r="V343" s="3" t="n"/>
+      <c r="W343" s="3" t="n"/>
+      <c r="X343" s="3" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="3" t="n"/>
@@ -8939,6 +9708,8 @@
       <c r="T344" s="3" t="n"/>
       <c r="U344" s="3" t="n"/>
       <c r="V344" s="3" t="n"/>
+      <c r="W344" s="3" t="n"/>
+      <c r="X344" s="3" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="3" t="n"/>
@@ -8963,6 +9734,8 @@
       <c r="T345" s="3" t="n"/>
       <c r="U345" s="3" t="n"/>
       <c r="V345" s="3" t="n"/>
+      <c r="W345" s="3" t="n"/>
+      <c r="X345" s="3" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="3" t="n"/>
@@ -8987,6 +9760,8 @@
       <c r="T346" s="3" t="n"/>
       <c r="U346" s="3" t="n"/>
       <c r="V346" s="3" t="n"/>
+      <c r="W346" s="3" t="n"/>
+      <c r="X346" s="3" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="3" t="n"/>
@@ -9011,6 +9786,8 @@
       <c r="T347" s="3" t="n"/>
       <c r="U347" s="3" t="n"/>
       <c r="V347" s="3" t="n"/>
+      <c r="W347" s="3" t="n"/>
+      <c r="X347" s="3" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="3" t="n"/>
@@ -9035,6 +9812,8 @@
       <c r="T348" s="3" t="n"/>
       <c r="U348" s="3" t="n"/>
       <c r="V348" s="3" t="n"/>
+      <c r="W348" s="3" t="n"/>
+      <c r="X348" s="3" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="3" t="n"/>
@@ -9059,6 +9838,8 @@
       <c r="T349" s="3" t="n"/>
       <c r="U349" s="3" t="n"/>
       <c r="V349" s="3" t="n"/>
+      <c r="W349" s="3" t="n"/>
+      <c r="X349" s="3" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="3" t="n"/>
@@ -9083,6 +9864,8 @@
       <c r="T350" s="3" t="n"/>
       <c r="U350" s="3" t="n"/>
       <c r="V350" s="3" t="n"/>
+      <c r="W350" s="3" t="n"/>
+      <c r="X350" s="3" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="3" t="n"/>
@@ -9107,6 +9890,8 @@
       <c r="T351" s="3" t="n"/>
       <c r="U351" s="3" t="n"/>
       <c r="V351" s="3" t="n"/>
+      <c r="W351" s="3" t="n"/>
+      <c r="X351" s="3" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="3" t="n"/>
@@ -9131,6 +9916,8 @@
       <c r="T352" s="3" t="n"/>
       <c r="U352" s="3" t="n"/>
       <c r="V352" s="3" t="n"/>
+      <c r="W352" s="3" t="n"/>
+      <c r="X352" s="3" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="3" t="n"/>
@@ -9155,6 +9942,8 @@
       <c r="T353" s="3" t="n"/>
       <c r="U353" s="3" t="n"/>
       <c r="V353" s="3" t="n"/>
+      <c r="W353" s="3" t="n"/>
+      <c r="X353" s="3" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="3" t="n"/>
@@ -9179,6 +9968,8 @@
       <c r="T354" s="3" t="n"/>
       <c r="U354" s="3" t="n"/>
       <c r="V354" s="3" t="n"/>
+      <c r="W354" s="3" t="n"/>
+      <c r="X354" s="3" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="3" t="n"/>
@@ -9203,6 +9994,8 @@
       <c r="T355" s="3" t="n"/>
       <c r="U355" s="3" t="n"/>
       <c r="V355" s="3" t="n"/>
+      <c r="W355" s="3" t="n"/>
+      <c r="X355" s="3" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="3" t="n"/>
@@ -9227,6 +10020,8 @@
       <c r="T356" s="3" t="n"/>
       <c r="U356" s="3" t="n"/>
       <c r="V356" s="3" t="n"/>
+      <c r="W356" s="3" t="n"/>
+      <c r="X356" s="3" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="3" t="n"/>
@@ -9251,6 +10046,8 @@
       <c r="T357" s="3" t="n"/>
       <c r="U357" s="3" t="n"/>
       <c r="V357" s="3" t="n"/>
+      <c r="W357" s="3" t="n"/>
+      <c r="X357" s="3" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="3" t="n"/>
@@ -9275,6 +10072,8 @@
       <c r="T358" s="3" t="n"/>
       <c r="U358" s="3" t="n"/>
       <c r="V358" s="3" t="n"/>
+      <c r="W358" s="3" t="n"/>
+      <c r="X358" s="3" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="3" t="n"/>
@@ -9299,6 +10098,8 @@
       <c r="T359" s="3" t="n"/>
       <c r="U359" s="3" t="n"/>
       <c r="V359" s="3" t="n"/>
+      <c r="W359" s="3" t="n"/>
+      <c r="X359" s="3" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="3" t="n"/>
@@ -9323,6 +10124,8 @@
       <c r="T360" s="3" t="n"/>
       <c r="U360" s="3" t="n"/>
       <c r="V360" s="3" t="n"/>
+      <c r="W360" s="3" t="n"/>
+      <c r="X360" s="3" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="3" t="n"/>
@@ -9347,6 +10150,8 @@
       <c r="T361" s="3" t="n"/>
       <c r="U361" s="3" t="n"/>
       <c r="V361" s="3" t="n"/>
+      <c r="W361" s="3" t="n"/>
+      <c r="X361" s="3" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="3" t="n"/>
@@ -9371,6 +10176,8 @@
       <c r="T362" s="3" t="n"/>
       <c r="U362" s="3" t="n"/>
       <c r="V362" s="3" t="n"/>
+      <c r="W362" s="3" t="n"/>
+      <c r="X362" s="3" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="3" t="n"/>
@@ -9395,6 +10202,8 @@
       <c r="T363" s="3" t="n"/>
       <c r="U363" s="3" t="n"/>
       <c r="V363" s="3" t="n"/>
+      <c r="W363" s="3" t="n"/>
+      <c r="X363" s="3" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="3" t="n"/>
@@ -9419,6 +10228,8 @@
       <c r="T364" s="3" t="n"/>
       <c r="U364" s="3" t="n"/>
       <c r="V364" s="3" t="n"/>
+      <c r="W364" s="3" t="n"/>
+      <c r="X364" s="3" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="3" t="n"/>
@@ -9443,6 +10254,8 @@
       <c r="T365" s="3" t="n"/>
       <c r="U365" s="3" t="n"/>
       <c r="V365" s="3" t="n"/>
+      <c r="W365" s="3" t="n"/>
+      <c r="X365" s="3" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="3" t="n"/>
@@ -9467,6 +10280,8 @@
       <c r="T366" s="3" t="n"/>
       <c r="U366" s="3" t="n"/>
       <c r="V366" s="3" t="n"/>
+      <c r="W366" s="3" t="n"/>
+      <c r="X366" s="3" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="3" t="n"/>
@@ -9491,6 +10306,8 @@
       <c r="T367" s="3" t="n"/>
       <c r="U367" s="3" t="n"/>
       <c r="V367" s="3" t="n"/>
+      <c r="W367" s="3" t="n"/>
+      <c r="X367" s="3" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="3" t="n"/>
@@ -9515,6 +10332,8 @@
       <c r="T368" s="3" t="n"/>
       <c r="U368" s="3" t="n"/>
       <c r="V368" s="3" t="n"/>
+      <c r="W368" s="3" t="n"/>
+      <c r="X368" s="3" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="3" t="n"/>
@@ -9539,6 +10358,8 @@
       <c r="T369" s="3" t="n"/>
       <c r="U369" s="3" t="n"/>
       <c r="V369" s="3" t="n"/>
+      <c r="W369" s="3" t="n"/>
+      <c r="X369" s="3" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="3" t="n"/>
@@ -9563,6 +10384,8 @@
       <c r="T370" s="3" t="n"/>
       <c r="U370" s="3" t="n"/>
       <c r="V370" s="3" t="n"/>
+      <c r="W370" s="3" t="n"/>
+      <c r="X370" s="3" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="3" t="n"/>
@@ -9587,6 +10410,8 @@
       <c r="T371" s="3" t="n"/>
       <c r="U371" s="3" t="n"/>
       <c r="V371" s="3" t="n"/>
+      <c r="W371" s="3" t="n"/>
+      <c r="X371" s="3" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="3" t="n"/>
@@ -9611,6 +10436,8 @@
       <c r="T372" s="3" t="n"/>
       <c r="U372" s="3" t="n"/>
       <c r="V372" s="3" t="n"/>
+      <c r="W372" s="3" t="n"/>
+      <c r="X372" s="3" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="3" t="n"/>
@@ -9635,6 +10462,8 @@
       <c r="T373" s="3" t="n"/>
       <c r="U373" s="3" t="n"/>
       <c r="V373" s="3" t="n"/>
+      <c r="W373" s="3" t="n"/>
+      <c r="X373" s="3" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="3" t="n"/>
@@ -9659,6 +10488,8 @@
       <c r="T374" s="3" t="n"/>
       <c r="U374" s="3" t="n"/>
       <c r="V374" s="3" t="n"/>
+      <c r="W374" s="3" t="n"/>
+      <c r="X374" s="3" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="3" t="n"/>
@@ -9683,6 +10514,8 @@
       <c r="T375" s="3" t="n"/>
       <c r="U375" s="3" t="n"/>
       <c r="V375" s="3" t="n"/>
+      <c r="W375" s="3" t="n"/>
+      <c r="X375" s="3" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="3" t="n"/>
@@ -9707,6 +10540,8 @@
       <c r="T376" s="3" t="n"/>
       <c r="U376" s="3" t="n"/>
       <c r="V376" s="3" t="n"/>
+      <c r="W376" s="3" t="n"/>
+      <c r="X376" s="3" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="3" t="n"/>
@@ -9731,6 +10566,8 @@
       <c r="T377" s="3" t="n"/>
       <c r="U377" s="3" t="n"/>
       <c r="V377" s="3" t="n"/>
+      <c r="W377" s="3" t="n"/>
+      <c r="X377" s="3" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="3" t="n"/>
@@ -9755,6 +10592,8 @@
       <c r="T378" s="3" t="n"/>
       <c r="U378" s="3" t="n"/>
       <c r="V378" s="3" t="n"/>
+      <c r="W378" s="3" t="n"/>
+      <c r="X378" s="3" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="3" t="n"/>
@@ -9779,6 +10618,8 @@
       <c r="T379" s="3" t="n"/>
       <c r="U379" s="3" t="n"/>
       <c r="V379" s="3" t="n"/>
+      <c r="W379" s="3" t="n"/>
+      <c r="X379" s="3" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="3" t="n"/>
@@ -9803,6 +10644,8 @@
       <c r="T380" s="3" t="n"/>
       <c r="U380" s="3" t="n"/>
       <c r="V380" s="3" t="n"/>
+      <c r="W380" s="3" t="n"/>
+      <c r="X380" s="3" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="3" t="n"/>
@@ -9827,6 +10670,8 @@
       <c r="T381" s="3" t="n"/>
       <c r="U381" s="3" t="n"/>
       <c r="V381" s="3" t="n"/>
+      <c r="W381" s="3" t="n"/>
+      <c r="X381" s="3" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="3" t="n"/>
@@ -9851,6 +10696,8 @@
       <c r="T382" s="3" t="n"/>
       <c r="U382" s="3" t="n"/>
       <c r="V382" s="3" t="n"/>
+      <c r="W382" s="3" t="n"/>
+      <c r="X382" s="3" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="3" t="n"/>
@@ -9875,6 +10722,8 @@
       <c r="T383" s="3" t="n"/>
       <c r="U383" s="3" t="n"/>
       <c r="V383" s="3" t="n"/>
+      <c r="W383" s="3" t="n"/>
+      <c r="X383" s="3" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="3" t="n"/>
@@ -9899,6 +10748,8 @@
       <c r="T384" s="3" t="n"/>
       <c r="U384" s="3" t="n"/>
       <c r="V384" s="3" t="n"/>
+      <c r="W384" s="3" t="n"/>
+      <c r="X384" s="3" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="3" t="n"/>
@@ -9923,6 +10774,8 @@
       <c r="T385" s="3" t="n"/>
       <c r="U385" s="3" t="n"/>
       <c r="V385" s="3" t="n"/>
+      <c r="W385" s="3" t="n"/>
+      <c r="X385" s="3" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="3" t="n"/>
@@ -9947,6 +10800,8 @@
       <c r="T386" s="3" t="n"/>
       <c r="U386" s="3" t="n"/>
       <c r="V386" s="3" t="n"/>
+      <c r="W386" s="3" t="n"/>
+      <c r="X386" s="3" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="3" t="n"/>
@@ -9971,6 +10826,8 @@
       <c r="T387" s="3" t="n"/>
       <c r="U387" s="3" t="n"/>
       <c r="V387" s="3" t="n"/>
+      <c r="W387" s="3" t="n"/>
+      <c r="X387" s="3" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="3" t="n"/>
@@ -9995,6 +10852,8 @@
       <c r="T388" s="3" t="n"/>
       <c r="U388" s="3" t="n"/>
       <c r="V388" s="3" t="n"/>
+      <c r="W388" s="3" t="n"/>
+      <c r="X388" s="3" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="3" t="n"/>
@@ -10019,6 +10878,8 @@
       <c r="T389" s="3" t="n"/>
       <c r="U389" s="3" t="n"/>
       <c r="V389" s="3" t="n"/>
+      <c r="W389" s="3" t="n"/>
+      <c r="X389" s="3" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="3" t="n"/>
@@ -10043,6 +10904,8 @@
       <c r="T390" s="3" t="n"/>
       <c r="U390" s="3" t="n"/>
       <c r="V390" s="3" t="n"/>
+      <c r="W390" s="3" t="n"/>
+      <c r="X390" s="3" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="3" t="n"/>
@@ -10067,6 +10930,8 @@
       <c r="T391" s="3" t="n"/>
       <c r="U391" s="3" t="n"/>
       <c r="V391" s="3" t="n"/>
+      <c r="W391" s="3" t="n"/>
+      <c r="X391" s="3" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="3" t="n"/>
@@ -10091,6 +10956,8 @@
       <c r="T392" s="3" t="n"/>
       <c r="U392" s="3" t="n"/>
       <c r="V392" s="3" t="n"/>
+      <c r="W392" s="3" t="n"/>
+      <c r="X392" s="3" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="3" t="n"/>
@@ -10115,6 +10982,8 @@
       <c r="T393" s="3" t="n"/>
       <c r="U393" s="3" t="n"/>
       <c r="V393" s="3" t="n"/>
+      <c r="W393" s="3" t="n"/>
+      <c r="X393" s="3" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="3" t="n"/>
@@ -10139,6 +11008,8 @@
       <c r="T394" s="3" t="n"/>
       <c r="U394" s="3" t="n"/>
       <c r="V394" s="3" t="n"/>
+      <c r="W394" s="3" t="n"/>
+      <c r="X394" s="3" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="3" t="n"/>
@@ -10163,6 +11034,8 @@
       <c r="T395" s="3" t="n"/>
       <c r="U395" s="3" t="n"/>
       <c r="V395" s="3" t="n"/>
+      <c r="W395" s="3" t="n"/>
+      <c r="X395" s="3" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="3" t="n"/>
@@ -10187,6 +11060,8 @@
       <c r="T396" s="3" t="n"/>
       <c r="U396" s="3" t="n"/>
       <c r="V396" s="3" t="n"/>
+      <c r="W396" s="3" t="n"/>
+      <c r="X396" s="3" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="3" t="n"/>
@@ -10211,6 +11086,8 @@
       <c r="T397" s="3" t="n"/>
       <c r="U397" s="3" t="n"/>
       <c r="V397" s="3" t="n"/>
+      <c r="W397" s="3" t="n"/>
+      <c r="X397" s="3" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="3" t="n"/>
@@ -10235,6 +11112,8 @@
       <c r="T398" s="3" t="n"/>
       <c r="U398" s="3" t="n"/>
       <c r="V398" s="3" t="n"/>
+      <c r="W398" s="3" t="n"/>
+      <c r="X398" s="3" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="3" t="n"/>
@@ -10259,6 +11138,8 @@
       <c r="T399" s="3" t="n"/>
       <c r="U399" s="3" t="n"/>
       <c r="V399" s="3" t="n"/>
+      <c r="W399" s="3" t="n"/>
+      <c r="X399" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -10481,7 +11362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A43"/>
+  <dimension ref="A1:A49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -10609,164 +11490,206 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • insight_en / insight_th ไม่บังคับเลย — ปกติกรอกแค่ insight_th อย่างเดียวก็พอ</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>คำอธิบายรายคอลัมน์</t>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ระบบจะโชว์เนื้อหานี้ให้ทั้งตอนสลับเป็นโหมด EN และ TH โดยอัตโนมัติ (fallback แบบเดียวกับคำอธิบาย)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  id           เว้นว่างได้ ระบบจะรันเลขต่อให้เอง เช่น d1-0043</t>
+          <t xml:space="preserve">  • ในเซลล์ Excel กด Alt+Enter เพื่อขึ้นบรรทัดใหม่ได้ ระบบจะคงการขึ้นบรรทัดนั้นไว้ตอนแสดงผล</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  domain       หมายเลขโดเมน 1-8 (จำเป็น)</t>
+          <t xml:space="preserve">  • โดเมนที่ยังไม่มีโจทย์เลยจะไม่โผล่ในหน้าเลือกโดเมนของเว็บ — พอมีแถวแรกของโดเมนนั้นเข้าไปก็จะขึ้นเอง</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  type         single หรือ multi เว้นว่าง = single</t>
-        </is>
-      </c>
+      <c r="A24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  q_en         คำถามภาษาอังกฤษ (จำเป็น)</t>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>คำอธิบายรายคอลัมน์</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  q_th         คำถามภาษาไทย</t>
+          <t xml:space="preserve">  id           เว้นว่างได้ ระบบจะรันเลขต่อให้เอง เช่น d1-0043</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  a_en         ตัวเลือก A อังกฤษ</t>
+          <t xml:space="preserve">  domain       หมายเลขโดเมน 1-8 (จำเป็น)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  a_th         ตัวเลือก A ไทย</t>
+          <t xml:space="preserve">  type         single หรือ multi เว้นว่าง = single</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  b_en         ตัวเลือก B อังกฤษ</t>
+          <t xml:space="preserve">  q_en         คำถามภาษาอังกฤษ (จำเป็น)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  b_th         ตัวเลือก B ไทย</t>
+          <t xml:space="preserve">  q_th         คำถามภาษาไทย</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  c_en         ตัวเลือก C อังกฤษ</t>
+          <t xml:space="preserve">  a_en         ตัวเลือก A อังกฤษ</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  c_th         ตัวเลือก C ไทย</t>
+          <t xml:space="preserve">  a_th         ตัวเลือก A ไทย</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  d_en         ตัวเลือก D อังกฤษ</t>
+          <t xml:space="preserve">  b_en         ตัวเลือก B อังกฤษ</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  d_th         ตัวเลือก D ไทย</t>
+          <t xml:space="preserve">  b_th         ตัวเลือก B ไทย</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  e_en         ตัวเลือก E (ถ้ามี)</t>
+          <t xml:space="preserve">  c_en         ตัวเลือก C อังกฤษ</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  e_th         ตัวเลือก E ไทย</t>
+          <t xml:space="preserve">  c_th         ตัวเลือก C ไทย</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  f_en         ตัวเลือก F (ถ้ามี)</t>
+          <t xml:space="preserve">  d_en         ตัวเลือก D อังกฤษ</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  f_th         ตัวเลือก F ไทย</t>
+          <t xml:space="preserve">  d_th         ตัวเลือก D ไทย</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  answer       เฉลย เช่น B หรือ "B,D" ถ้าตอบได้หลายข้อ (จำเป็น)</t>
+          <t xml:space="preserve">  e_en         ตัวเลือก E (ถ้ามี)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  explain_en   คำอธิบายภาษาอังกฤษ</t>
+          <t xml:space="preserve">  e_th         ตัวเลือก E ไทย</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  explain_th   คำอธิบายภาษาไทย</t>
+          <t xml:space="preserve">  f_en         ตัวเลือก F (ถ้ามี)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  tags         แท็ก คั่นด้วย ; เช่น risk;governance</t>
+          <t xml:space="preserve">  f_th         ตัวเลือก F ไทย</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  answer       เฉลย เช่น B หรือ "B,D" ถ้าตอบได้หลายข้อ (จำเป็น)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  explain_en   คำอธิบายภาษาอังกฤษ (ทำไมข้อนี้ถูก)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  explain_th   คำอธิบายภาษาไทย (ทำไมข้อนี้ถูก)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  insight_en   เพิ่มเติม/บทวิเคราะห์เชิงลึก อังกฤษ (ไม่บังคับ กด Alt+Enter ขึ้นบรรทัดใหม่ในเซลล์ได้)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  insight_th   เพิ่มเติม/บทวิเคราะห์เชิงลึก ไทย (ไม่บังคับ — ปกติกรอกแค่คอลัมน์นี้คอลัมน์เดียวก็พอ ระบบจะโชว์ให้ทั้งโหมด EN และ TH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  tags         แท็ก คั่นด้วย ; เช่น risk;governance</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t xml:space="preserve">  ref          อ้างอิง เช่น OSG ch.1</t>
         </is>

</xml_diff>